<commit_message>
Redesign: colour-coded timeline, city landmarks, done-ticks; Map opens the app directly
- Category colour code mirroring the workbook; per-city colour and line-art
  landmark on the hero and each sticky, collapsible day header; day strip;
  must-see / food / optional / travel filter chips; tick a stop done; 'up
  next' from China time during the trip.
- Map button now deep-links into the Amap app (iosamap:// / androidamap://)
  straight into transit directions using GCJ-02 coordinates for every
  landmark, hotel and station, with a web fallback if the app is missing;
  Apple Maps offered on iPhone. Replaces the slow uri.amap.com hand-off.
- Generator pulls the workbook from the shared iCloud link first; local
  copy is the fallback. Picks up the new Impression West Lake show on Day 2.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/itinerary.xlsx
+++ b/tools/itinerary.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mameedd-my.sharepoint.com/personal/jitwei_tan_mamee_com_my/Documents/Documents/Copilot/Created/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jitwei/Library/Mobile Documents/com~apple~CloudDocs/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="668" documentId="11_97678BFFD66160F5F3CE075E0DFED605AB16B636" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0ECEE288-F3FB-2E45-BB56-DCD28EF40EE2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2406BDD5-9AE0-784C-A160-D80875152CF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-6080" yWindow="-21000" windowWidth="38400" windowHeight="21000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1457" uniqueCount="981">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1463" uniqueCount="987">
   <si>
     <r>
       <rPr>
@@ -8544,9 +8544,6 @@
     </r>
   </si>
   <si>
-    <t>19:15–20:00</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="10"/>
@@ -8583,9 +8580,6 @@
       </rPr>
       <t>清河坊</t>
     </r>
-  </si>
-  <si>
-    <t>Silk, tea, fans, scissors, snacks.</t>
   </si>
   <si>
     <r>
@@ -14505,6 +14499,30 @@
   </si>
   <si>
     <t>World's most beautiful bookstore' in a converted car park. Pairs with 颐和路; go before noon.</t>
+  </si>
+  <si>
+    <t>19:30–20:30</t>
+  </si>
+  <si>
+    <t>MUST-SEE: 印象西湖《最忆是杭州》 Impression West Lake</t>
+  </si>
+  <si>
+    <t>MANDATORY — outdoor water-stage show on West Lake itself (Zhang Yimou). ~50–60 min. Arrive 30–60 min early; seating by zone. Outdoor — may adjust in rain. Book ahead.</t>
+  </si>
+  <si>
+    <t>¥238–880 · 岳湖</t>
+  </si>
+  <si>
+    <t>西湖区北山路82号 (岳湖景区, 岳庙对面)</t>
+  </si>
+  <si>
+    <t>18:50–19:30</t>
+  </si>
+  <si>
+    <t>Quick browse — head to 岳湖 by 19:00 for the show.</t>
+  </si>
+  <si>
+    <t>20:45–21:30</t>
   </si>
 </sst>
 </file>
@@ -15058,7 +15076,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="206">
+  <cellXfs count="207">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -15504,6 +15522,33 @@
     <xf numFmtId="0" fontId="7" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -15529,33 +15574,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -15585,6 +15603,42 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -15602,42 +15656,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -15667,6 +15685,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -16158,7 +16179,7 @@
   <sheetPr>
     <tabColor rgb="FFC55A11"/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -16170,24 +16191,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="160" t="s">
+      <c r="A1" s="151" t="s">
         <v>396</v>
       </c>
-      <c r="B1" s="161"/>
-      <c r="C1" s="161"/>
-      <c r="D1" s="161"/>
-      <c r="E1" s="161"/>
-      <c r="F1" s="162"/>
+      <c r="B1" s="152"/>
+      <c r="C1" s="152"/>
+      <c r="D1" s="152"/>
+      <c r="E1" s="152"/>
+      <c r="F1" s="153"/>
     </row>
     <row r="2" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A2" s="163" t="s">
+      <c r="A2" s="154" t="s">
         <v>397</v>
       </c>
-      <c r="B2" s="164"/>
-      <c r="C2" s="164"/>
-      <c r="D2" s="164"/>
-      <c r="E2" s="164"/>
-      <c r="F2" s="165"/>
+      <c r="B2" s="155"/>
+      <c r="C2" s="155"/>
+      <c r="D2" s="155"/>
+      <c r="E2" s="155"/>
+      <c r="F2" s="156"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1">
       <c r="A3" s="77" t="s">
@@ -16210,14 +16231,14 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A4" s="166" t="s">
+      <c r="A4" s="157" t="s">
         <v>403</v>
       </c>
-      <c r="B4" s="167"/>
-      <c r="C4" s="167"/>
-      <c r="D4" s="167"/>
-      <c r="E4" s="167"/>
-      <c r="F4" s="168"/>
+      <c r="B4" s="158"/>
+      <c r="C4" s="158"/>
+      <c r="D4" s="158"/>
+      <c r="E4" s="158"/>
+      <c r="F4" s="159"/>
     </row>
     <row r="5" spans="1:6" ht="25.5" customHeight="1">
       <c r="A5" s="98" t="s">
@@ -16420,14 +16441,14 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A15" s="166" t="s">
+      <c r="A15" s="157" t="s">
         <v>452</v>
       </c>
-      <c r="B15" s="167"/>
-      <c r="C15" s="167"/>
-      <c r="D15" s="167"/>
-      <c r="E15" s="167"/>
-      <c r="F15" s="168"/>
+      <c r="B15" s="158"/>
+      <c r="C15" s="158"/>
+      <c r="D15" s="158"/>
+      <c r="E15" s="158"/>
+      <c r="F15" s="159"/>
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="101" t="s">
@@ -16674,1885 +16695,1905 @@
         <v>453</v>
       </c>
       <c r="B28" s="57" t="s">
+        <v>984</v>
+      </c>
+      <c r="C28" s="33" t="s">
         <v>507</v>
       </c>
-      <c r="C28" s="33" t="s">
+      <c r="D28" s="33" t="s">
+        <v>985</v>
+      </c>
+      <c r="E28" s="33" t="s">
         <v>508</v>
-      </c>
-      <c r="D28" s="33" t="s">
-        <v>509</v>
-      </c>
-      <c r="E28" s="33" t="s">
-        <v>510</v>
       </c>
       <c r="F28" s="117" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A29" s="107" t="s">
+    <row r="29" spans="1:6" ht="42">
+      <c r="A29" s="102" t="s">
         <v>453</v>
       </c>
-      <c r="B29" s="64" t="s">
-        <v>439</v>
-      </c>
-      <c r="C29" s="36" t="s">
+      <c r="B29" s="57" t="s">
+        <v>979</v>
+      </c>
+      <c r="C29" s="33" t="s">
+        <v>980</v>
+      </c>
+      <c r="D29" s="33" t="s">
+        <v>981</v>
+      </c>
+      <c r="E29" s="33" t="s">
+        <v>982</v>
+      </c>
+      <c r="F29" s="117" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="25" customHeight="1">
+      <c r="A30" s="107" t="s">
+        <v>453</v>
+      </c>
+      <c r="B30" s="64" t="s">
+        <v>986</v>
+      </c>
+      <c r="C30" s="36" t="s">
+        <v>509</v>
+      </c>
+      <c r="D30" s="36" t="s">
+        <v>510</v>
+      </c>
+      <c r="E30" s="36" t="s">
         <v>511</v>
       </c>
-      <c r="D29" s="36" t="s">
+      <c r="F30" s="122" t="s">
         <v>512</v>
       </c>
-      <c r="E29" s="36" t="s">
-        <v>513</v>
-      </c>
-      <c r="F29" s="122" t="s">
+    </row>
+    <row r="31" spans="1:6" ht="21.75" customHeight="1">
+      <c r="A31" s="101" t="s">
+        <v>453</v>
+      </c>
+      <c r="B31" s="206" t="s">
+        <v>968</v>
+      </c>
+      <c r="C31" s="10" t="s">
         <v>514</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A30" s="101" t="s">
-        <v>453</v>
-      </c>
-      <c r="B30" s="56" t="s">
+      <c r="D31" s="10"/>
+      <c r="E31" s="10" t="s">
+        <v>451</v>
+      </c>
+      <c r="F31" s="116" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A32" s="157" t="s">
         <v>515</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="B32" s="158"/>
+      <c r="C32" s="158"/>
+      <c r="D32" s="158"/>
+      <c r="E32" s="158"/>
+      <c r="F32" s="159"/>
+    </row>
+    <row r="33" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A33" s="101" t="s">
         <v>516</v>
       </c>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10" t="s">
-        <v>451</v>
-      </c>
-      <c r="F30" s="116" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A31" s="166" t="s">
+      <c r="B33" s="56" t="s">
         <v>517</v>
       </c>
-      <c r="B31" s="167"/>
-      <c r="C31" s="167"/>
-      <c r="D31" s="167"/>
-      <c r="E31" s="167"/>
-      <c r="F31" s="168"/>
-    </row>
-    <row r="32" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A32" s="101" t="s">
+      <c r="C33" s="10" t="s">
+        <v>455</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>518</v>
       </c>
-      <c r="B32" s="56" t="s">
-        <v>519</v>
-      </c>
-      <c r="C32" s="10" t="s">
-        <v>455</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>520</v>
-      </c>
-      <c r="E32" s="10" t="s">
+      <c r="E33" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F32" s="116" t="s">
+      <c r="F33" s="116" t="s">
         <v>28</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A33" s="105" t="s">
-        <v>518</v>
-      </c>
-      <c r="B33" s="60" t="s">
-        <v>521</v>
-      </c>
-      <c r="C33" s="61" t="s">
-        <v>522</v>
-      </c>
-      <c r="D33" s="61" t="s">
-        <v>523</v>
-      </c>
-      <c r="E33" s="61" t="s">
-        <v>524</v>
-      </c>
-      <c r="F33" s="120" t="s">
-        <v>525</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="25.5" customHeight="1">
       <c r="A34" s="105" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="B34" s="60" t="s">
+        <v>519</v>
+      </c>
+      <c r="C34" s="61" t="s">
+        <v>520</v>
+      </c>
+      <c r="D34" s="61" t="s">
+        <v>521</v>
+      </c>
+      <c r="E34" s="61" t="s">
+        <v>522</v>
+      </c>
+      <c r="F34" s="120" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A35" s="105" t="s">
+        <v>516</v>
+      </c>
+      <c r="B35" s="60" t="s">
+        <v>524</v>
+      </c>
+      <c r="C35" s="61" t="s">
+        <v>525</v>
+      </c>
+      <c r="D35" s="61" t="s">
         <v>526</v>
       </c>
-      <c r="C34" s="61" t="s">
+      <c r="E35" s="61" t="s">
         <v>527</v>
       </c>
-      <c r="D34" s="61" t="s">
+      <c r="F35" s="120" t="s">
         <v>528</v>
       </c>
-      <c r="E34" s="61" t="s">
+    </row>
+    <row r="36" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A36" s="104" t="s">
+        <v>516</v>
+      </c>
+      <c r="B36" s="59" t="s">
         <v>529</v>
       </c>
-      <c r="F34" s="120" t="s">
+      <c r="C36" s="47" t="s">
         <v>530</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A35" s="104" t="s">
-        <v>518</v>
-      </c>
-      <c r="B35" s="59" t="s">
+      <c r="D36" s="47" t="s">
         <v>531</v>
       </c>
-      <c r="C35" s="47" t="s">
+      <c r="E36" s="47" t="s">
+        <v>460</v>
+      </c>
+      <c r="F36" s="119" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A37" s="99" t="s">
+        <v>516</v>
+      </c>
+      <c r="B37" s="54" t="s">
         <v>532</v>
       </c>
-      <c r="D35" s="47" t="s">
+      <c r="C37" s="15" t="s">
         <v>533</v>
       </c>
-      <c r="E35" s="47" t="s">
-        <v>460</v>
-      </c>
-      <c r="F35" s="119" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A36" s="99" t="s">
-        <v>518</v>
-      </c>
-      <c r="B36" s="54" t="s">
+      <c r="D37" s="15" t="s">
         <v>534</v>
       </c>
-      <c r="C36" s="15" t="s">
+      <c r="E37" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="F37" s="85" t="s">
         <v>535</v>
       </c>
-      <c r="D36" s="15" t="s">
+    </row>
+    <row r="38" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A38" s="105" t="s">
+        <v>516</v>
+      </c>
+      <c r="B38" s="60" t="s">
         <v>536</v>
       </c>
-      <c r="E36" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="F36" s="85" t="s">
+      <c r="C38" s="61" t="s">
         <v>537</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A37" s="105" t="s">
-        <v>518</v>
-      </c>
-      <c r="B37" s="60" t="s">
+      <c r="D38" s="61" t="s">
         <v>538</v>
       </c>
-      <c r="C37" s="61" t="s">
+      <c r="E38" s="61" t="s">
+        <v>527</v>
+      </c>
+      <c r="F38" s="120" t="s">
         <v>539</v>
       </c>
-      <c r="D37" s="61" t="s">
+    </row>
+    <row r="39" spans="1:6" ht="30" customHeight="1">
+      <c r="A39" s="103" t="s">
+        <v>516</v>
+      </c>
+      <c r="B39" s="58" t="s">
         <v>540</v>
       </c>
-      <c r="E37" s="61" t="s">
-        <v>529</v>
-      </c>
-      <c r="F37" s="120" t="s">
+      <c r="C39" s="39" t="s">
         <v>541</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A38" s="103" t="s">
-        <v>518</v>
-      </c>
-      <c r="B38" s="58" t="s">
+      <c r="D39" s="39" t="s">
         <v>542</v>
       </c>
-      <c r="C38" s="39" t="s">
+      <c r="E39" s="39" t="s">
         <v>543</v>
       </c>
-      <c r="D38" s="39" t="s">
+      <c r="F39" s="118" t="s">
         <v>544</v>
       </c>
-      <c r="E38" s="39" t="s">
+    </row>
+    <row r="40" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A40" s="108" t="s">
+        <v>516</v>
+      </c>
+      <c r="B40" s="89" t="s">
+        <v>940</v>
+      </c>
+      <c r="C40" s="90" t="s">
+        <v>941</v>
+      </c>
+      <c r="D40" s="90" t="s">
+        <v>942</v>
+      </c>
+      <c r="E40" s="90" t="s">
+        <v>943</v>
+      </c>
+      <c r="F40" s="123" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A41" s="102" t="s">
+        <v>516</v>
+      </c>
+      <c r="B41" s="57" t="s">
+        <v>662</v>
+      </c>
+      <c r="C41" s="33" t="s">
         <v>545</v>
       </c>
-      <c r="F38" s="118" t="s">
+      <c r="D41" s="33" t="s">
         <v>546</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="30" customHeight="1">
-      <c r="A39" s="108" t="s">
-        <v>518</v>
-      </c>
-      <c r="B39" s="89" t="s">
-        <v>942</v>
-      </c>
-      <c r="C39" s="90" t="s">
-        <v>943</v>
-      </c>
-      <c r="D39" s="90" t="s">
-        <v>944</v>
-      </c>
-      <c r="E39" s="90" t="s">
-        <v>945</v>
-      </c>
-      <c r="F39" s="123" t="s">
-        <v>946</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A40" s="102" t="s">
-        <v>518</v>
-      </c>
-      <c r="B40" s="57" t="s">
-        <v>664</v>
-      </c>
-      <c r="C40" s="33" t="s">
+      <c r="E41" s="35" t="s">
         <v>547</v>
       </c>
-      <c r="D40" s="33" t="s">
+      <c r="F41" s="117" t="s">
         <v>548</v>
       </c>
-      <c r="E40" s="35" t="s">
+    </row>
+    <row r="42" spans="1:6" ht="30" customHeight="1">
+      <c r="A42" s="106" t="s">
+        <v>516</v>
+      </c>
+      <c r="B42" s="63" t="s">
+        <v>962</v>
+      </c>
+      <c r="C42" s="20" t="s">
         <v>549</v>
       </c>
-      <c r="F40" s="117" t="s">
+      <c r="D42" s="20" t="s">
         <v>550</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A41" s="106" t="s">
-        <v>518</v>
-      </c>
-      <c r="B41" s="63" t="s">
-        <v>964</v>
-      </c>
-      <c r="C41" s="20" t="s">
+      <c r="E42" s="20" t="s">
         <v>551</v>
       </c>
-      <c r="D41" s="20" t="s">
+      <c r="F42" s="121" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A43" s="105" t="s">
+        <v>516</v>
+      </c>
+      <c r="B43" s="60" t="s">
+        <v>497</v>
+      </c>
+      <c r="C43" s="61" t="s">
         <v>552</v>
       </c>
-      <c r="E41" s="20" t="s">
+      <c r="D43" s="61" t="s">
         <v>553</v>
       </c>
-      <c r="F41" s="121" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="30" customHeight="1">
-      <c r="A42" s="105" t="s">
-        <v>518</v>
-      </c>
-      <c r="B42" s="60" t="s">
-        <v>497</v>
-      </c>
-      <c r="C42" s="61" t="s">
+      <c r="E43" s="61" t="s">
         <v>554</v>
       </c>
-      <c r="D42" s="61" t="s">
+      <c r="F43" s="120" t="s">
         <v>555</v>
       </c>
-      <c r="E42" s="61" t="s">
+    </row>
+    <row r="44" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A44" s="103" t="s">
+        <v>516</v>
+      </c>
+      <c r="B44" s="58" t="s">
         <v>556</v>
       </c>
-      <c r="F42" s="120" t="s">
+      <c r="C44" s="39" t="s">
         <v>557</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A43" s="103" t="s">
-        <v>518</v>
-      </c>
-      <c r="B43" s="58" t="s">
+      <c r="D44" s="39" t="s">
         <v>558</v>
       </c>
-      <c r="C43" s="39" t="s">
+      <c r="E44" s="39" t="s">
         <v>559</v>
       </c>
-      <c r="D43" s="39" t="s">
+      <c r="F44" s="118" t="s">
         <v>560</v>
       </c>
-      <c r="E43" s="39" t="s">
+    </row>
+    <row r="45" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A45" s="98" t="s">
+        <v>516</v>
+      </c>
+      <c r="B45" s="53" t="s">
         <v>561</v>
       </c>
-      <c r="F43" s="118" t="s">
+      <c r="C45" s="5" t="s">
         <v>562</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A44" s="98" t="s">
-        <v>518</v>
-      </c>
-      <c r="B44" s="53" t="s">
+      <c r="D45" s="5" t="s">
         <v>563</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="E45" s="5" t="s">
         <v>564</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="F45" s="86" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A46" s="101" t="s">
+        <v>516</v>
+      </c>
+      <c r="B46" s="56" t="s">
         <v>565</v>
       </c>
-      <c r="E44" s="5" t="s">
+      <c r="C46" s="10" t="s">
         <v>566</v>
       </c>
-      <c r="F44" s="86" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A45" s="101" t="s">
-        <v>518</v>
-      </c>
-      <c r="B45" s="56" t="s">
+      <c r="D46" s="10" t="s">
         <v>567</v>
       </c>
-      <c r="C45" s="10" t="s">
+      <c r="E46" s="10" t="s">
+        <v>451</v>
+      </c>
+      <c r="F46" s="116" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A47" s="109" t="s">
+        <v>516</v>
+      </c>
+      <c r="B47" s="65" t="s">
         <v>568</v>
       </c>
-      <c r="D45" s="10" t="s">
+      <c r="C47" s="42" t="s">
         <v>569</v>
       </c>
-      <c r="E45" s="10" t="s">
-        <v>451</v>
-      </c>
-      <c r="F45" s="116" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A46" s="109" t="s">
-        <v>518</v>
-      </c>
-      <c r="B46" s="65" t="s">
+      <c r="D47" s="42" t="s">
         <v>570</v>
       </c>
-      <c r="C46" s="42" t="s">
+      <c r="E47" s="42" t="s">
         <v>571</v>
       </c>
-      <c r="D46" s="42" t="s">
+      <c r="F47" s="124" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="21.75" customHeight="1">
+      <c r="A48" s="103" t="s">
+        <v>516</v>
+      </c>
+      <c r="B48" s="58" t="s">
+        <v>568</v>
+      </c>
+      <c r="C48" s="39" t="s">
         <v>572</v>
       </c>
-      <c r="E46" s="42" t="s">
+      <c r="D48" s="39" t="s">
         <v>573</v>
       </c>
-      <c r="F46" s="124" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A47" s="103" t="s">
-        <v>518</v>
-      </c>
-      <c r="B47" s="58" t="s">
-        <v>570</v>
-      </c>
-      <c r="C47" s="39" t="s">
+      <c r="E48" s="39" t="s">
+        <v>571</v>
+      </c>
+      <c r="F48" s="118" t="s">
         <v>574</v>
       </c>
-      <c r="D47" s="39" t="s">
+    </row>
+    <row r="49" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A49" s="160" t="s">
         <v>575</v>
       </c>
-      <c r="E47" s="39" t="s">
-        <v>573</v>
-      </c>
-      <c r="F47" s="118" t="s">
+      <c r="B49" s="161"/>
+      <c r="C49" s="161"/>
+      <c r="D49" s="161"/>
+      <c r="E49" s="161"/>
+      <c r="F49" s="162"/>
+    </row>
+    <row r="50" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A50" s="101" t="s">
         <v>576</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A48" s="151" t="s">
+      <c r="B50" s="56" t="s">
+        <v>517</v>
+      </c>
+      <c r="C50" s="10" t="s">
         <v>577</v>
       </c>
-      <c r="B48" s="152"/>
-      <c r="C48" s="152"/>
-      <c r="D48" s="152"/>
-      <c r="E48" s="152"/>
-      <c r="F48" s="153"/>
-    </row>
-    <row r="49" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A49" s="101" t="s">
+      <c r="D50" s="10" t="s">
         <v>578</v>
       </c>
-      <c r="B49" s="56" t="s">
-        <v>519</v>
-      </c>
-      <c r="C49" s="10" t="s">
+      <c r="E50" s="10" t="s">
         <v>579</v>
       </c>
-      <c r="D49" s="10" t="s">
-        <v>580</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>581</v>
-      </c>
-      <c r="F49" s="116" t="s">
+      <c r="F50" s="116" t="s">
         <v>28</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A50" s="100" t="s">
-        <v>578</v>
-      </c>
-      <c r="B50" s="55" t="s">
-        <v>582</v>
-      </c>
-      <c r="C50" s="50" t="s">
-        <v>583</v>
-      </c>
-      <c r="D50" s="50" t="s">
-        <v>584</v>
-      </c>
-      <c r="E50" s="50" t="s">
-        <v>585</v>
-      </c>
-      <c r="F50" s="115" t="s">
-        <v>586</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="25.5" customHeight="1">
       <c r="A51" s="100" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B51" s="55" t="s">
+        <v>580</v>
+      </c>
+      <c r="C51" s="50" t="s">
+        <v>581</v>
+      </c>
+      <c r="D51" s="50" t="s">
+        <v>582</v>
+      </c>
+      <c r="E51" s="50" t="s">
+        <v>583</v>
+      </c>
+      <c r="F51" s="115" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="30" customHeight="1">
+      <c r="A52" s="100" t="s">
+        <v>576</v>
+      </c>
+      <c r="B52" s="55" t="s">
+        <v>585</v>
+      </c>
+      <c r="C52" s="50" t="s">
+        <v>586</v>
+      </c>
+      <c r="D52" s="50" t="s">
         <v>587</v>
       </c>
-      <c r="C51" s="50" t="s">
+      <c r="E52" s="50" t="s">
         <v>588</v>
       </c>
-      <c r="D51" s="50" t="s">
+      <c r="F52" s="115" t="s">
         <v>589</v>
       </c>
-      <c r="E51" s="50" t="s">
+    </row>
+    <row r="53" spans="1:6" ht="30" customHeight="1">
+      <c r="A53" s="101" t="s">
+        <v>576</v>
+      </c>
+      <c r="B53" s="56" t="s">
         <v>590</v>
       </c>
-      <c r="F51" s="115" t="s">
+      <c r="C53" s="10" t="s">
         <v>591</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" ht="30" customHeight="1">
-      <c r="A52" s="101" t="s">
-        <v>578</v>
-      </c>
-      <c r="B52" s="56" t="s">
+      <c r="D53" s="10" t="s">
         <v>592</v>
       </c>
-      <c r="C52" s="10" t="s">
+      <c r="E53" s="10" t="s">
+        <v>433</v>
+      </c>
+      <c r="F53" s="116" t="s">
         <v>593</v>
       </c>
-      <c r="D52" s="10" t="s">
+    </row>
+    <row r="54" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A54" s="99" t="s">
+        <v>576</v>
+      </c>
+      <c r="B54" s="54" t="s">
         <v>594</v>
       </c>
-      <c r="E52" s="10" t="s">
-        <v>433</v>
-      </c>
-      <c r="F52" s="116" t="s">
+      <c r="C54" s="15" t="s">
         <v>595</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" ht="30" customHeight="1">
-      <c r="A53" s="99" t="s">
-        <v>578</v>
-      </c>
-      <c r="B53" s="54" t="s">
+      <c r="D54" s="25" t="s">
         <v>596</v>
       </c>
-      <c r="C53" s="15" t="s">
-        <v>597</v>
-      </c>
-      <c r="D53" s="25" t="s">
-        <v>598</v>
-      </c>
-      <c r="E53" s="15" t="s">
+      <c r="E54" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="F53" s="85" t="s">
+      <c r="F54" s="85" t="s">
         <v>318</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A54" s="105" t="s">
-        <v>578</v>
-      </c>
-      <c r="B54" s="60" t="s">
-        <v>599</v>
-      </c>
-      <c r="C54" s="61" t="s">
-        <v>600</v>
-      </c>
-      <c r="D54" s="61" t="s">
-        <v>601</v>
-      </c>
-      <c r="E54" s="61" t="s">
-        <v>529</v>
-      </c>
-      <c r="F54" s="120" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="25.5" customHeight="1">
       <c r="A55" s="105" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B55" s="60" t="s">
+        <v>597</v>
+      </c>
+      <c r="C55" s="61" t="s">
+        <v>598</v>
+      </c>
+      <c r="D55" s="61" t="s">
+        <v>599</v>
+      </c>
+      <c r="E55" s="61" t="s">
+        <v>527</v>
+      </c>
+      <c r="F55" s="120" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A56" s="105" t="s">
+        <v>576</v>
+      </c>
+      <c r="B56" s="60" t="s">
+        <v>600</v>
+      </c>
+      <c r="C56" s="61" t="s">
+        <v>601</v>
+      </c>
+      <c r="D56" s="61" t="s">
         <v>602</v>
       </c>
-      <c r="C55" s="61" t="s">
+      <c r="E56" s="61" t="s">
         <v>603</v>
       </c>
-      <c r="D55" s="61" t="s">
+      <c r="F56" s="120" t="s">
         <v>604</v>
       </c>
-      <c r="E55" s="61" t="s">
+    </row>
+    <row r="57" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A57" s="106" t="s">
+        <v>576</v>
+      </c>
+      <c r="B57" s="63" t="s">
         <v>605</v>
       </c>
-      <c r="F55" s="120" t="s">
+      <c r="C57" s="20" t="s">
         <v>606</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A56" s="106" t="s">
-        <v>578</v>
-      </c>
-      <c r="B56" s="63" t="s">
+      <c r="D57" s="20" t="s">
         <v>607</v>
       </c>
-      <c r="C56" s="20" t="s">
+      <c r="E57" s="20" t="s">
         <v>608</v>
       </c>
-      <c r="D56" s="20" t="s">
+      <c r="F57" s="121" t="s">
         <v>609</v>
       </c>
-      <c r="E56" s="20" t="s">
+    </row>
+    <row r="58" spans="1:6" ht="45" customHeight="1">
+      <c r="A58" s="105" t="s">
+        <v>576</v>
+      </c>
+      <c r="B58" s="60" t="s">
         <v>610</v>
       </c>
-      <c r="F56" s="121" t="s">
+      <c r="C58" s="61" t="s">
         <v>611</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A57" s="105" t="s">
-        <v>578</v>
-      </c>
-      <c r="B57" s="60" t="s">
+      <c r="D58" s="61" t="s">
         <v>612</v>
       </c>
-      <c r="C57" s="61" t="s">
+      <c r="E58" s="61" t="s">
+        <v>603</v>
+      </c>
+      <c r="F58" s="120" t="s">
         <v>613</v>
       </c>
-      <c r="D57" s="61" t="s">
+    </row>
+    <row r="59" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A59" s="110" t="s">
+        <v>576</v>
+      </c>
+      <c r="B59" s="91" t="s">
+        <v>963</v>
+      </c>
+      <c r="C59" s="92" t="s">
+        <v>945</v>
+      </c>
+      <c r="D59" s="92" t="s">
+        <v>946</v>
+      </c>
+      <c r="E59" s="92" t="s">
+        <v>947</v>
+      </c>
+      <c r="F59" s="125" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="30" customHeight="1">
+      <c r="A60" s="105" t="s">
+        <v>576</v>
+      </c>
+      <c r="B60" s="60" t="s">
+        <v>618</v>
+      </c>
+      <c r="C60" s="61" t="s">
         <v>614</v>
       </c>
-      <c r="E57" s="61" t="s">
-        <v>605</v>
-      </c>
-      <c r="F57" s="120" t="s">
+      <c r="D60" s="61" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" ht="45" customHeight="1">
-      <c r="A58" s="110" t="s">
-        <v>578</v>
-      </c>
-      <c r="B58" s="91" t="s">
+      <c r="E60" s="61" t="s">
+        <v>616</v>
+      </c>
+      <c r="F60" s="120" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="30" customHeight="1">
+      <c r="A61" s="107" t="s">
+        <v>576</v>
+      </c>
+      <c r="B61" s="64" t="s">
+        <v>964</v>
+      </c>
+      <c r="C61" s="36" t="s">
+        <v>619</v>
+      </c>
+      <c r="D61" s="36" t="s">
+        <v>620</v>
+      </c>
+      <c r="E61" s="36" t="s">
+        <v>621</v>
+      </c>
+      <c r="F61" s="122" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A62" s="109" t="s">
+        <v>576</v>
+      </c>
+      <c r="B62" s="65" t="s">
         <v>965</v>
       </c>
-      <c r="C58" s="92" t="s">
-        <v>947</v>
-      </c>
-      <c r="D58" s="92" t="s">
-        <v>948</v>
-      </c>
-      <c r="E58" s="92" t="s">
+      <c r="C62" s="42" t="s">
+        <v>623</v>
+      </c>
+      <c r="D62" s="44" t="s">
+        <v>624</v>
+      </c>
+      <c r="E62" s="42" t="s">
+        <v>625</v>
+      </c>
+      <c r="F62" s="124" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="21.75" customHeight="1">
+      <c r="A63" s="101" t="s">
+        <v>576</v>
+      </c>
+      <c r="B63" s="128" t="s">
+        <v>968</v>
+      </c>
+      <c r="C63" s="10" t="s">
+        <v>628</v>
+      </c>
+      <c r="D63" s="10"/>
+      <c r="E63" s="10" t="s">
+        <v>629</v>
+      </c>
+      <c r="F63" s="116" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A64" s="160" t="s">
+        <v>630</v>
+      </c>
+      <c r="B64" s="161"/>
+      <c r="C64" s="161"/>
+      <c r="D64" s="161"/>
+      <c r="E64" s="161"/>
+      <c r="F64" s="162"/>
+    </row>
+    <row r="65" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A65" s="101" t="s">
+        <v>631</v>
+      </c>
+      <c r="B65" s="56" t="s">
+        <v>517</v>
+      </c>
+      <c r="C65" s="10" t="s">
+        <v>632</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>633</v>
+      </c>
+      <c r="E65" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F65" s="116" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="30" customHeight="1">
+      <c r="A66" s="105" t="s">
+        <v>631</v>
+      </c>
+      <c r="B66" s="60" t="s">
+        <v>634</v>
+      </c>
+      <c r="C66" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="D66" s="62" t="s">
+        <v>636</v>
+      </c>
+      <c r="E66" s="61" t="s">
+        <v>637</v>
+      </c>
+      <c r="F66" s="120" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="30" customHeight="1">
+      <c r="A67" s="108" t="s">
+        <v>631</v>
+      </c>
+      <c r="B67" s="89" t="s">
         <v>949</v>
       </c>
-      <c r="F58" s="125" t="s">
+      <c r="C67" s="90" t="s">
         <v>950</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A59" s="105" t="s">
-        <v>578</v>
-      </c>
-      <c r="B59" s="60" t="s">
-        <v>620</v>
-      </c>
-      <c r="C59" s="61" t="s">
-        <v>616</v>
-      </c>
-      <c r="D59" s="61" t="s">
-        <v>617</v>
-      </c>
-      <c r="E59" s="61" t="s">
-        <v>618</v>
-      </c>
-      <c r="F59" s="120" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="30" customHeight="1">
-      <c r="A60" s="107" t="s">
-        <v>578</v>
-      </c>
-      <c r="B60" s="64" t="s">
+      <c r="D67" s="90" t="s">
+        <v>951</v>
+      </c>
+      <c r="E67" s="90" t="s">
+        <v>952</v>
+      </c>
+      <c r="F67" s="123" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="30" customHeight="1">
+      <c r="A68" s="103" t="s">
+        <v>631</v>
+      </c>
+      <c r="B68" s="58" t="s">
         <v>966</v>
       </c>
-      <c r="C60" s="36" t="s">
-        <v>621</v>
-      </c>
-      <c r="D60" s="36" t="s">
-        <v>622</v>
-      </c>
-      <c r="E60" s="36" t="s">
-        <v>623</v>
-      </c>
-      <c r="F60" s="122" t="s">
-        <v>624</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" ht="30" customHeight="1">
-      <c r="A61" s="109" t="s">
-        <v>578</v>
-      </c>
-      <c r="B61" s="65" t="s">
-        <v>967</v>
-      </c>
-      <c r="C61" s="42" t="s">
-        <v>625</v>
-      </c>
-      <c r="D61" s="44" t="s">
-        <v>626</v>
-      </c>
-      <c r="E61" s="42" t="s">
-        <v>627</v>
-      </c>
-      <c r="F61" s="124" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A62" s="101" t="s">
-        <v>578</v>
-      </c>
-      <c r="B62" s="128" t="s">
-        <v>970</v>
-      </c>
-      <c r="C62" s="10" t="s">
-        <v>630</v>
-      </c>
-      <c r="D62" s="10"/>
-      <c r="E62" s="10" t="s">
+      <c r="C68" s="39" t="s">
+        <v>639</v>
+      </c>
+      <c r="D68" s="39" t="s">
+        <v>640</v>
+      </c>
+      <c r="E68" s="39" t="s">
+        <v>641</v>
+      </c>
+      <c r="F68" s="118" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A69" s="104" t="s">
         <v>631</v>
       </c>
-      <c r="F62" s="116" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A63" s="151" t="s">
-        <v>632</v>
-      </c>
-      <c r="B63" s="152"/>
-      <c r="C63" s="152"/>
-      <c r="D63" s="152"/>
-      <c r="E63" s="152"/>
-      <c r="F63" s="153"/>
-    </row>
-    <row r="64" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A64" s="101" t="s">
-        <v>633</v>
-      </c>
-      <c r="B64" s="56" t="s">
-        <v>519</v>
-      </c>
-      <c r="C64" s="10" t="s">
-        <v>634</v>
-      </c>
-      <c r="D64" s="10" t="s">
-        <v>635</v>
-      </c>
-      <c r="E64" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F64" s="116" t="s">
+      <c r="B69" s="59" t="s">
+        <v>475</v>
+      </c>
+      <c r="C69" s="47" t="s">
+        <v>643</v>
+      </c>
+      <c r="D69" s="47" t="s">
+        <v>644</v>
+      </c>
+      <c r="E69" s="47" t="s">
+        <v>645</v>
+      </c>
+      <c r="F69" s="119" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A70" s="105" t="s">
+        <v>631</v>
+      </c>
+      <c r="B70" s="60" t="s">
+        <v>647</v>
+      </c>
+      <c r="C70" s="61" t="s">
+        <v>648</v>
+      </c>
+      <c r="D70" s="61" t="s">
+        <v>649</v>
+      </c>
+      <c r="E70" s="61" t="s">
+        <v>650</v>
+      </c>
+      <c r="F70" s="120" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="30" customHeight="1">
+      <c r="A71" s="98" t="s">
+        <v>631</v>
+      </c>
+      <c r="B71" s="53" t="s">
+        <v>652</v>
+      </c>
+      <c r="C71" s="5" t="s">
+        <v>653</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>654</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="F71" s="86" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="30" customHeight="1">
+      <c r="A72" s="103" t="s">
+        <v>631</v>
+      </c>
+      <c r="B72" s="58" t="s">
+        <v>657</v>
+      </c>
+      <c r="C72" s="39" t="s">
+        <v>658</v>
+      </c>
+      <c r="D72" s="39" t="s">
+        <v>659</v>
+      </c>
+      <c r="E72" s="39" t="s">
+        <v>660</v>
+      </c>
+      <c r="F72" s="118" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="30" customHeight="1">
+      <c r="A73" s="105" t="s">
+        <v>631</v>
+      </c>
+      <c r="B73" s="60" t="s">
+        <v>662</v>
+      </c>
+      <c r="C73" s="61" t="s">
+        <v>663</v>
+      </c>
+      <c r="D73" s="61" t="s">
+        <v>664</v>
+      </c>
+      <c r="E73" s="61" t="s">
+        <v>665</v>
+      </c>
+      <c r="F73" s="120" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A74" s="104" t="s">
+        <v>631</v>
+      </c>
+      <c r="B74" s="59" t="s">
+        <v>667</v>
+      </c>
+      <c r="C74" s="47" t="s">
+        <v>668</v>
+      </c>
+      <c r="D74" s="47" t="s">
+        <v>669</v>
+      </c>
+      <c r="E74" s="47" t="s">
+        <v>660</v>
+      </c>
+      <c r="F74" s="119" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="30" customHeight="1">
+      <c r="A75" s="106" t="s">
+        <v>631</v>
+      </c>
+      <c r="B75" s="63" t="s">
+        <v>671</v>
+      </c>
+      <c r="C75" s="20" t="s">
+        <v>672</v>
+      </c>
+      <c r="D75" s="20" t="s">
+        <v>673</v>
+      </c>
+      <c r="E75" s="20" t="s">
+        <v>674</v>
+      </c>
+      <c r="F75" s="121" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="30" customHeight="1">
+      <c r="A76" s="102" t="s">
+        <v>631</v>
+      </c>
+      <c r="B76" s="57" t="s">
+        <v>676</v>
+      </c>
+      <c r="C76" s="33" t="s">
+        <v>677</v>
+      </c>
+      <c r="D76" s="33" t="s">
+        <v>678</v>
+      </c>
+      <c r="E76" s="33" t="s">
+        <v>679</v>
+      </c>
+      <c r="F76" s="117" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A65" s="105" t="s">
-        <v>633</v>
-      </c>
-      <c r="B65" s="60" t="s">
-        <v>636</v>
-      </c>
-      <c r="C65" s="61" t="s">
-        <v>637</v>
-      </c>
-      <c r="D65" s="62" t="s">
-        <v>638</v>
-      </c>
-      <c r="E65" s="61" t="s">
-        <v>639</v>
-      </c>
-      <c r="F65" s="120" t="s">
-        <v>640</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="30" customHeight="1">
-      <c r="A66" s="108" t="s">
-        <v>633</v>
-      </c>
-      <c r="B66" s="89" t="s">
-        <v>951</v>
-      </c>
-      <c r="C66" s="90" t="s">
-        <v>952</v>
-      </c>
-      <c r="D66" s="90" t="s">
-        <v>953</v>
-      </c>
-      <c r="E66" s="90" t="s">
-        <v>954</v>
-      </c>
-      <c r="F66" s="123" t="s">
-        <v>955</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" ht="30" customHeight="1">
-      <c r="A67" s="103" t="s">
-        <v>633</v>
-      </c>
-      <c r="B67" s="58" t="s">
-        <v>968</v>
-      </c>
-      <c r="C67" s="39" t="s">
-        <v>641</v>
-      </c>
-      <c r="D67" s="39" t="s">
-        <v>642</v>
-      </c>
-      <c r="E67" s="39" t="s">
-        <v>643</v>
-      </c>
-      <c r="F67" s="118" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" ht="30" customHeight="1">
-      <c r="A68" s="104" t="s">
-        <v>633</v>
-      </c>
-      <c r="B68" s="59" t="s">
-        <v>475</v>
-      </c>
-      <c r="C68" s="47" t="s">
-        <v>645</v>
-      </c>
-      <c r="D68" s="47" t="s">
-        <v>646</v>
-      </c>
-      <c r="E68" s="47" t="s">
-        <v>647</v>
-      </c>
-      <c r="F68" s="119" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A69" s="105" t="s">
-        <v>633</v>
-      </c>
-      <c r="B69" s="60" t="s">
-        <v>649</v>
-      </c>
-      <c r="C69" s="61" t="s">
-        <v>650</v>
-      </c>
-      <c r="D69" s="61" t="s">
-        <v>651</v>
-      </c>
-      <c r="E69" s="61" t="s">
-        <v>652</v>
-      </c>
-      <c r="F69" s="120" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A70" s="98" t="s">
-        <v>633</v>
-      </c>
-      <c r="B70" s="53" t="s">
-        <v>654</v>
-      </c>
-      <c r="C70" s="5" t="s">
-        <v>655</v>
-      </c>
-      <c r="D70" s="5" t="s">
-        <v>656</v>
-      </c>
-      <c r="E70" s="5" t="s">
-        <v>657</v>
-      </c>
-      <c r="F70" s="86" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" ht="30" customHeight="1">
-      <c r="A71" s="103" t="s">
-        <v>633</v>
-      </c>
-      <c r="B71" s="58" t="s">
-        <v>659</v>
-      </c>
-      <c r="C71" s="39" t="s">
-        <v>660</v>
-      </c>
-      <c r="D71" s="39" t="s">
-        <v>661</v>
-      </c>
-      <c r="E71" s="39" t="s">
-        <v>662</v>
-      </c>
-      <c r="F71" s="118" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" ht="30" customHeight="1">
-      <c r="A72" s="105" t="s">
-        <v>633</v>
-      </c>
-      <c r="B72" s="60" t="s">
-        <v>664</v>
-      </c>
-      <c r="C72" s="61" t="s">
-        <v>665</v>
-      </c>
-      <c r="D72" s="61" t="s">
-        <v>666</v>
-      </c>
-      <c r="E72" s="61" t="s">
-        <v>667</v>
-      </c>
-      <c r="F72" s="120" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" ht="30" customHeight="1">
-      <c r="A73" s="104" t="s">
-        <v>633</v>
-      </c>
-      <c r="B73" s="59" t="s">
-        <v>669</v>
-      </c>
-      <c r="C73" s="47" t="s">
-        <v>670</v>
-      </c>
-      <c r="D73" s="47" t="s">
-        <v>671</v>
-      </c>
-      <c r="E73" s="47" t="s">
-        <v>662</v>
-      </c>
-      <c r="F73" s="119" t="s">
-        <v>672</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A74" s="106" t="s">
-        <v>633</v>
-      </c>
-      <c r="B74" s="63" t="s">
-        <v>673</v>
-      </c>
-      <c r="C74" s="20" t="s">
-        <v>674</v>
-      </c>
-      <c r="D74" s="20" t="s">
-        <v>675</v>
-      </c>
-      <c r="E74" s="20" t="s">
-        <v>676</v>
-      </c>
-      <c r="F74" s="121" t="s">
-        <v>677</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" ht="30" customHeight="1">
-      <c r="A75" s="102" t="s">
-        <v>633</v>
-      </c>
-      <c r="B75" s="57" t="s">
-        <v>678</v>
-      </c>
-      <c r="C75" s="33" t="s">
-        <v>679</v>
-      </c>
-      <c r="D75" s="33" t="s">
+    <row r="77" spans="1:6" ht="30" customHeight="1">
+      <c r="A77" s="107" t="s">
+        <v>631</v>
+      </c>
+      <c r="B77" s="64" t="s">
+        <v>561</v>
+      </c>
+      <c r="C77" s="36" t="s">
         <v>680</v>
       </c>
-      <c r="E75" s="33" t="s">
+      <c r="D77" s="36" t="s">
         <v>681</v>
       </c>
-      <c r="F75" s="117" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" ht="30" customHeight="1">
-      <c r="A76" s="107" t="s">
-        <v>633</v>
-      </c>
-      <c r="B76" s="64" t="s">
-        <v>563</v>
-      </c>
-      <c r="C76" s="36" t="s">
-        <v>682</v>
-      </c>
-      <c r="D76" s="36" t="s">
-        <v>683</v>
-      </c>
-      <c r="E76" s="36" t="s">
+      <c r="E77" s="36" t="s">
         <v>210</v>
       </c>
-      <c r="F76" s="122" t="s">
+      <c r="F77" s="122" t="s">
         <v>241</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" ht="30" customHeight="1">
-      <c r="A77" s="101" t="s">
-        <v>633</v>
-      </c>
-      <c r="B77" s="56" t="s">
-        <v>684</v>
-      </c>
-      <c r="C77" s="10" t="s">
-        <v>685</v>
-      </c>
-      <c r="D77" s="10" t="s">
-        <v>686</v>
-      </c>
-      <c r="E77" s="10" t="s">
-        <v>561</v>
-      </c>
-      <c r="F77" s="116" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="25.5" customHeight="1">
       <c r="A78" s="101" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="B78" s="56" t="s">
+        <v>682</v>
+      </c>
+      <c r="C78" s="10" t="s">
+        <v>683</v>
+      </c>
+      <c r="D78" s="10" t="s">
+        <v>684</v>
+      </c>
+      <c r="E78" s="10" t="s">
+        <v>559</v>
+      </c>
+      <c r="F78" s="116" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="30" customHeight="1">
+      <c r="A79" s="101" t="s">
+        <v>631</v>
+      </c>
+      <c r="B79" s="56" t="s">
+        <v>627</v>
+      </c>
+      <c r="C79" s="10" t="s">
+        <v>685</v>
+      </c>
+      <c r="D79" s="10" t="s">
+        <v>686</v>
+      </c>
+      <c r="E79" s="10" t="s">
         <v>629</v>
       </c>
-      <c r="C78" s="10" t="s">
-        <v>687</v>
-      </c>
-      <c r="D78" s="10" t="s">
-        <v>688</v>
-      </c>
-      <c r="E78" s="10" t="s">
-        <v>631</v>
-      </c>
-      <c r="F78" s="116" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" ht="30" customHeight="1">
-      <c r="A79" s="103" t="s">
-        <v>633</v>
-      </c>
-      <c r="B79" s="58" t="s">
-        <v>570</v>
-      </c>
-      <c r="C79" s="39" t="s">
-        <v>689</v>
-      </c>
-      <c r="D79" s="39" t="s">
-        <v>690</v>
-      </c>
-      <c r="E79" s="39" t="s">
-        <v>573</v>
-      </c>
-      <c r="F79" s="118" t="s">
-        <v>691</v>
+      <c r="F79" s="116" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="30" customHeight="1">
       <c r="A80" s="103" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="B80" s="58" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="C80" s="39" t="s">
-        <v>692</v>
+        <v>687</v>
       </c>
       <c r="D80" s="39" t="s">
-        <v>693</v>
+        <v>688</v>
       </c>
       <c r="E80" s="39" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="F80" s="118" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="30" customHeight="1">
       <c r="A81" s="103" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="B81" s="58" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="C81" s="39" t="s">
+        <v>690</v>
+      </c>
+      <c r="D81" s="39" t="s">
+        <v>691</v>
+      </c>
+      <c r="E81" s="39" t="s">
+        <v>571</v>
+      </c>
+      <c r="F81" s="118" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="30" customHeight="1">
+      <c r="A82" s="103" t="s">
+        <v>631</v>
+      </c>
+      <c r="B82" s="58" t="s">
+        <v>568</v>
+      </c>
+      <c r="C82" s="39" t="s">
+        <v>693</v>
+      </c>
+      <c r="D82" s="39" t="s">
+        <v>694</v>
+      </c>
+      <c r="E82" s="39" t="s">
+        <v>571</v>
+      </c>
+      <c r="F82" s="118" t="s">
         <v>695</v>
       </c>
-      <c r="D81" s="39" t="s">
+    </row>
+    <row r="83" spans="1:6" ht="21.75" customHeight="1">
+      <c r="A83" s="108" t="s">
+        <v>631</v>
+      </c>
+      <c r="B83" s="89" t="s">
+        <v>568</v>
+      </c>
+      <c r="C83" s="90" t="s">
+        <v>954</v>
+      </c>
+      <c r="D83" s="95" t="s">
+        <v>955</v>
+      </c>
+      <c r="E83" s="90" t="s">
+        <v>956</v>
+      </c>
+      <c r="F83" s="123" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A84" s="163" t="s">
         <v>696</v>
       </c>
-      <c r="E81" s="39" t="s">
-        <v>573</v>
-      </c>
-      <c r="F81" s="118" t="s">
+      <c r="B84" s="164"/>
+      <c r="C84" s="164"/>
+      <c r="D84" s="164"/>
+      <c r="E84" s="164"/>
+      <c r="F84" s="165"/>
+    </row>
+    <row r="85" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A85" s="101" t="s">
         <v>697</v>
       </c>
-    </row>
-    <row r="82" spans="1:6" ht="30" customHeight="1">
-      <c r="A82" s="108" t="s">
-        <v>633</v>
-      </c>
-      <c r="B82" s="89" t="s">
-        <v>570</v>
-      </c>
-      <c r="C82" s="90" t="s">
-        <v>956</v>
-      </c>
-      <c r="D82" s="95" t="s">
-        <v>957</v>
-      </c>
-      <c r="E82" s="90" t="s">
-        <v>958</v>
-      </c>
-      <c r="F82" s="123" t="s">
-        <v>959</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A83" s="154" t="s">
+      <c r="B85" s="56" t="s">
+        <v>517</v>
+      </c>
+      <c r="C85" s="10" t="s">
         <v>698</v>
       </c>
-      <c r="B83" s="155"/>
-      <c r="C83" s="155"/>
-      <c r="D83" s="155"/>
-      <c r="E83" s="155"/>
-      <c r="F83" s="156"/>
-    </row>
-    <row r="84" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A84" s="101" t="s">
-        <v>699</v>
-      </c>
-      <c r="B84" s="56" t="s">
-        <v>519</v>
-      </c>
-      <c r="C84" s="10" t="s">
-        <v>700</v>
-      </c>
-      <c r="D84" s="10"/>
-      <c r="E84" s="10" t="s">
-        <v>581</v>
-      </c>
-      <c r="F84" s="116" t="s">
+      <c r="D85" s="10"/>
+      <c r="E85" s="10" t="s">
+        <v>579</v>
+      </c>
+      <c r="F85" s="116" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A85" s="100" t="s">
-        <v>699</v>
-      </c>
-      <c r="B85" s="55" t="s">
-        <v>582</v>
-      </c>
-      <c r="C85" s="50" t="s">
-        <v>701</v>
-      </c>
-      <c r="D85" s="50" t="s">
-        <v>702</v>
-      </c>
-      <c r="E85" s="50" t="s">
-        <v>585</v>
-      </c>
-      <c r="F85" s="115" t="s">
-        <v>703</v>
       </c>
     </row>
     <row r="86" spans="1:6" ht="25.5" customHeight="1">
       <c r="A86" s="100" t="s">
+        <v>697</v>
+      </c>
+      <c r="B86" s="55" t="s">
+        <v>580</v>
+      </c>
+      <c r="C86" s="50" t="s">
         <v>699</v>
       </c>
-      <c r="B86" s="55" t="s">
-        <v>587</v>
-      </c>
-      <c r="C86" s="50" t="s">
+      <c r="D86" s="50" t="s">
+        <v>700</v>
+      </c>
+      <c r="E86" s="50" t="s">
+        <v>583</v>
+      </c>
+      <c r="F86" s="115" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="30" customHeight="1">
+      <c r="A87" s="100" t="s">
+        <v>697</v>
+      </c>
+      <c r="B87" s="55" t="s">
+        <v>585</v>
+      </c>
+      <c r="C87" s="50" t="s">
+        <v>702</v>
+      </c>
+      <c r="D87" s="50" t="s">
+        <v>703</v>
+      </c>
+      <c r="E87" s="50" t="s">
+        <v>588</v>
+      </c>
+      <c r="F87" s="115" t="s">
         <v>704</v>
       </c>
-      <c r="D86" s="50" t="s">
+    </row>
+    <row r="88" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A88" s="101" t="s">
+        <v>697</v>
+      </c>
+      <c r="B88" s="56" t="s">
+        <v>590</v>
+      </c>
+      <c r="C88" s="10" t="s">
         <v>705</v>
       </c>
-      <c r="E86" s="50" t="s">
-        <v>590</v>
-      </c>
-      <c r="F86" s="115" t="s">
+      <c r="D88" s="10" t="s">
         <v>706</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" ht="30" customHeight="1">
-      <c r="A87" s="101" t="s">
-        <v>699</v>
-      </c>
-      <c r="B87" s="56" t="s">
-        <v>592</v>
-      </c>
-      <c r="C87" s="10" t="s">
+      <c r="E88" s="10" t="s">
         <v>707</v>
       </c>
-      <c r="D87" s="10" t="s">
+      <c r="F88" s="116" t="s">
         <v>708</v>
       </c>
-      <c r="E87" s="10" t="s">
+    </row>
+    <row r="89" spans="1:6" ht="30" customHeight="1">
+      <c r="A89" s="99" t="s">
+        <v>697</v>
+      </c>
+      <c r="B89" s="54" t="s">
+        <v>594</v>
+      </c>
+      <c r="C89" s="15" t="s">
         <v>709</v>
       </c>
-      <c r="F87" s="116" t="s">
+      <c r="D89" s="15" t="s">
         <v>710</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A88" s="99" t="s">
-        <v>699</v>
-      </c>
-      <c r="B88" s="54" t="s">
-        <v>596</v>
-      </c>
-      <c r="C88" s="15" t="s">
-        <v>711</v>
-      </c>
-      <c r="D88" s="15" t="s">
-        <v>712</v>
-      </c>
-      <c r="E88" s="15" t="s">
+      <c r="E89" s="15" t="s">
         <v>220</v>
       </c>
-      <c r="F88" s="85" t="s">
+      <c r="F89" s="85" t="s">
         <v>131</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" ht="30" customHeight="1">
-      <c r="A89" s="105" t="s">
-        <v>699</v>
-      </c>
-      <c r="B89" s="60" t="s">
-        <v>713</v>
-      </c>
-      <c r="C89" s="61" t="s">
-        <v>714</v>
-      </c>
-      <c r="D89" s="61" t="s">
-        <v>715</v>
-      </c>
-      <c r="E89" s="61" t="s">
-        <v>716</v>
-      </c>
-      <c r="F89" s="120" t="s">
-        <v>717</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="30" customHeight="1">
       <c r="A90" s="105" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="B90" s="60" t="s">
-        <v>718</v>
+        <v>711</v>
       </c>
       <c r="C90" s="61" t="s">
-        <v>719</v>
+        <v>712</v>
       </c>
       <c r="D90" s="61" t="s">
-        <v>720</v>
+        <v>713</v>
       </c>
       <c r="E90" s="61" t="s">
-        <v>639</v>
+        <v>714</v>
       </c>
       <c r="F90" s="120" t="s">
-        <v>721</v>
+        <v>715</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="25.5" customHeight="1">
       <c r="A91" s="105" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="B91" s="60" t="s">
+        <v>716</v>
+      </c>
+      <c r="C91" s="61" t="s">
+        <v>717</v>
+      </c>
+      <c r="D91" s="61" t="s">
+        <v>718</v>
+      </c>
+      <c r="E91" s="61" t="s">
+        <v>637</v>
+      </c>
+      <c r="F91" s="120" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A92" s="105" t="s">
+        <v>697</v>
+      </c>
+      <c r="B92" s="60" t="s">
+        <v>720</v>
+      </c>
+      <c r="C92" s="61" t="s">
+        <v>721</v>
+      </c>
+      <c r="D92" s="61" t="s">
         <v>722</v>
       </c>
-      <c r="C91" s="61" t="s">
+      <c r="E92" s="61" t="s">
         <v>723</v>
       </c>
-      <c r="D91" s="61" t="s">
+      <c r="F92" s="120" t="s">
         <v>724</v>
       </c>
-      <c r="E91" s="61" t="s">
+    </row>
+    <row r="93" spans="1:6" ht="30" customHeight="1">
+      <c r="A93" s="106" t="s">
+        <v>697</v>
+      </c>
+      <c r="B93" s="63" t="s">
         <v>725</v>
       </c>
-      <c r="F91" s="120" t="s">
+      <c r="C93" s="20" t="s">
         <v>726</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A92" s="106" t="s">
-        <v>699</v>
-      </c>
-      <c r="B92" s="63" t="s">
+      <c r="D93" s="20" t="s">
         <v>727</v>
       </c>
-      <c r="C92" s="20" t="s">
+      <c r="E93" s="20" t="s">
         <v>728</v>
       </c>
-      <c r="D92" s="20" t="s">
+      <c r="F93" s="121" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" ht="30" customHeight="1">
+      <c r="A94" s="105" t="s">
+        <v>697</v>
+      </c>
+      <c r="B94" s="60" t="s">
         <v>729</v>
       </c>
-      <c r="E92" s="20" t="s">
+      <c r="C94" s="61" t="s">
         <v>730</v>
       </c>
-      <c r="F92" s="121" t="s">
+      <c r="D94" s="61" t="s">
+        <v>731</v>
+      </c>
+      <c r="E94" s="61" t="s">
+        <v>111</v>
+      </c>
+      <c r="F94" s="120" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="30" customHeight="1">
-      <c r="A93" s="105" t="s">
-        <v>699</v>
-      </c>
-      <c r="B93" s="60" t="s">
-        <v>731</v>
-      </c>
-      <c r="C93" s="61" t="s">
+    <row r="95" spans="1:6" ht="30" customHeight="1">
+      <c r="A95" s="109" t="s">
+        <v>697</v>
+      </c>
+      <c r="B95" s="65" t="s">
         <v>732</v>
       </c>
-      <c r="D93" s="61" t="s">
+      <c r="C95" s="42" t="s">
         <v>733</v>
       </c>
-      <c r="E93" s="61" t="s">
-        <v>111</v>
-      </c>
-      <c r="F93" s="120" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" ht="30" customHeight="1">
-      <c r="A94" s="109" t="s">
-        <v>699</v>
-      </c>
-      <c r="B94" s="65" t="s">
+      <c r="D95" s="42" t="s">
         <v>734</v>
       </c>
-      <c r="C94" s="42" t="s">
+      <c r="E95" s="42" t="s">
         <v>735</v>
       </c>
-      <c r="D94" s="42" t="s">
+      <c r="F95" s="124" t="s">
         <v>736</v>
       </c>
-      <c r="E94" s="42" t="s">
+    </row>
+    <row r="96" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A96" s="111" t="s">
+        <v>697</v>
+      </c>
+      <c r="B96" s="93" t="s">
+        <v>958</v>
+      </c>
+      <c r="C96" s="94" t="s">
+        <v>959</v>
+      </c>
+      <c r="D96" s="94" t="s">
+        <v>960</v>
+      </c>
+      <c r="E96" s="94" t="s">
+        <v>961</v>
+      </c>
+      <c r="F96" s="126" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" ht="45" customHeight="1">
+      <c r="A97" s="101" t="s">
+        <v>697</v>
+      </c>
+      <c r="B97" s="128" t="s">
+        <v>968</v>
+      </c>
+      <c r="C97" s="10" t="s">
+        <v>967</v>
+      </c>
+      <c r="D97" s="10"/>
+      <c r="E97" s="10" t="s">
+        <v>629</v>
+      </c>
+      <c r="F97" s="116" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="30" customHeight="1">
+      <c r="A98" s="102" t="s">
+        <v>697</v>
+      </c>
+      <c r="B98" s="57" t="s">
         <v>737</v>
       </c>
-      <c r="F94" s="124" t="s">
+      <c r="C98" s="33" t="s">
         <v>738</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" ht="30" customHeight="1">
-      <c r="A95" s="111" t="s">
-        <v>699</v>
-      </c>
-      <c r="B95" s="93" t="s">
-        <v>960</v>
-      </c>
-      <c r="C95" s="94" t="s">
-        <v>961</v>
-      </c>
-      <c r="D95" s="94" t="s">
-        <v>962</v>
-      </c>
-      <c r="E95" s="94" t="s">
-        <v>963</v>
-      </c>
-      <c r="F95" s="126" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A96" s="101" t="s">
-        <v>699</v>
-      </c>
-      <c r="B96" s="128" t="s">
-        <v>970</v>
-      </c>
-      <c r="C96" s="10" t="s">
-        <v>969</v>
-      </c>
-      <c r="D96" s="10"/>
-      <c r="E96" s="10" t="s">
-        <v>631</v>
-      </c>
-      <c r="F96" s="116" t="s">
-        <v>710</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" ht="45" customHeight="1">
-      <c r="A97" s="102" t="s">
-        <v>699</v>
-      </c>
-      <c r="B97" s="57" t="s">
+      <c r="D98" s="33" t="s">
         <v>739</v>
       </c>
-      <c r="C97" s="33" t="s">
+      <c r="E98" s="33" t="s">
+        <v>559</v>
+      </c>
+      <c r="F98" s="117" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="21.75" customHeight="1">
+      <c r="A99" s="103" t="s">
+        <v>697</v>
+      </c>
+      <c r="B99" s="58" t="s">
+        <v>737</v>
+      </c>
+      <c r="C99" s="39" t="s">
         <v>740</v>
       </c>
-      <c r="D97" s="33" t="s">
+      <c r="D99" s="39" t="s">
         <v>741</v>
       </c>
-      <c r="E97" s="33" t="s">
-        <v>561</v>
-      </c>
-      <c r="F97" s="117" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" ht="30" customHeight="1">
-      <c r="A98" s="103" t="s">
-        <v>699</v>
-      </c>
-      <c r="B98" s="58" t="s">
-        <v>739</v>
-      </c>
-      <c r="C98" s="39" t="s">
+      <c r="E99" s="39" t="s">
+        <v>559</v>
+      </c>
+      <c r="F99" s="118" t="s">
         <v>742</v>
       </c>
-      <c r="D98" s="39" t="s">
+    </row>
+    <row r="100" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A100" s="163" t="s">
         <v>743</v>
       </c>
-      <c r="E98" s="39" t="s">
-        <v>561</v>
-      </c>
-      <c r="F98" s="118" t="s">
+      <c r="B100" s="164"/>
+      <c r="C100" s="164"/>
+      <c r="D100" s="164"/>
+      <c r="E100" s="164"/>
+      <c r="F100" s="165"/>
+    </row>
+    <row r="101" spans="1:6" ht="30" customHeight="1">
+      <c r="A101" s="101" t="s">
         <v>744</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A99" s="154" t="s">
+      <c r="B101" s="56" t="s">
+        <v>517</v>
+      </c>
+      <c r="C101" s="10" t="s">
+        <v>632</v>
+      </c>
+      <c r="D101" s="10" t="s">
         <v>745</v>
       </c>
-      <c r="B99" s="155"/>
-      <c r="C99" s="155"/>
-      <c r="D99" s="155"/>
-      <c r="E99" s="155"/>
-      <c r="F99" s="156"/>
-    </row>
-    <row r="100" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A100" s="101" t="s">
-        <v>746</v>
-      </c>
-      <c r="B100" s="56" t="s">
-        <v>519</v>
-      </c>
-      <c r="C100" s="10" t="s">
-        <v>634</v>
-      </c>
-      <c r="D100" s="10" t="s">
-        <v>747</v>
-      </c>
-      <c r="E100" s="10" t="s">
+      <c r="E101" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F100" s="116" t="s">
+      <c r="F101" s="116" t="s">
         <v>37</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" ht="30" customHeight="1">
-      <c r="A101" s="105" t="s">
-        <v>746</v>
-      </c>
-      <c r="B101" s="60" t="s">
-        <v>521</v>
-      </c>
-      <c r="C101" s="61" t="s">
-        <v>748</v>
-      </c>
-      <c r="D101" s="61" t="s">
-        <v>749</v>
-      </c>
-      <c r="E101" s="61" t="s">
-        <v>524</v>
-      </c>
-      <c r="F101" s="120" t="s">
-        <v>750</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="30" customHeight="1">
       <c r="A102" s="105" t="s">
+        <v>744</v>
+      </c>
+      <c r="B102" s="60" t="s">
+        <v>519</v>
+      </c>
+      <c r="C102" s="61" t="s">
         <v>746</v>
       </c>
-      <c r="B102" s="60" t="s">
-        <v>751</v>
-      </c>
-      <c r="C102" s="61" t="s">
-        <v>752</v>
-      </c>
       <c r="D102" s="61" t="s">
-        <v>753</v>
+        <v>747</v>
       </c>
       <c r="E102" s="61" t="s">
-        <v>754</v>
+        <v>522</v>
       </c>
       <c r="F102" s="120" t="s">
-        <v>755</v>
+        <v>748</v>
       </c>
     </row>
     <row r="103" spans="1:6" ht="45" customHeight="1">
       <c r="A103" s="105" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="B103" s="60" t="s">
-        <v>649</v>
+        <v>749</v>
       </c>
       <c r="C103" s="61" t="s">
+        <v>750</v>
+      </c>
+      <c r="D103" s="61" t="s">
+        <v>751</v>
+      </c>
+      <c r="E103" s="61" t="s">
+        <v>752</v>
+      </c>
+      <c r="F103" s="120" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A104" s="105" t="s">
+        <v>744</v>
+      </c>
+      <c r="B104" s="60" t="s">
+        <v>647</v>
+      </c>
+      <c r="C104" s="61" t="s">
+        <v>754</v>
+      </c>
+      <c r="D104" s="61" t="s">
+        <v>755</v>
+      </c>
+      <c r="E104" s="61" t="s">
         <v>756</v>
       </c>
-      <c r="D103" s="61" t="s">
+      <c r="F104" s="120" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A105" s="98" t="s">
+        <v>744</v>
+      </c>
+      <c r="B105" s="53" t="s">
         <v>757</v>
       </c>
-      <c r="E103" s="61" t="s">
+      <c r="C105" s="5" t="s">
         <v>758</v>
       </c>
-      <c r="F103" s="120" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A104" s="98" t="s">
-        <v>746</v>
-      </c>
-      <c r="B104" s="53" t="s">
+      <c r="D105" s="5" t="s">
         <v>759</v>
       </c>
-      <c r="C104" s="5" t="s">
+      <c r="E105" s="5" t="s">
         <v>760</v>
       </c>
-      <c r="D104" s="5" t="s">
+      <c r="F105" s="86" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" ht="30" customHeight="1">
+      <c r="A106" s="102" t="s">
+        <v>744</v>
+      </c>
+      <c r="B106" s="57" t="s">
+        <v>657</v>
+      </c>
+      <c r="C106" s="33" t="s">
         <v>761</v>
       </c>
-      <c r="E104" s="5" t="s">
+      <c r="D106" s="33" t="s">
         <v>762</v>
       </c>
-      <c r="F104" s="86" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A105" s="102" t="s">
-        <v>746</v>
-      </c>
-      <c r="B105" s="57" t="s">
-        <v>659</v>
-      </c>
-      <c r="C105" s="33" t="s">
+      <c r="E106" s="33" t="s">
         <v>763</v>
       </c>
-      <c r="D105" s="33" t="s">
+      <c r="F106" s="117" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A107" s="105" t="s">
+        <v>744</v>
+      </c>
+      <c r="B107" s="60" t="s">
         <v>764</v>
       </c>
-      <c r="E105" s="33" t="s">
+      <c r="C107" s="61" t="s">
         <v>765</v>
       </c>
-      <c r="F105" s="117" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" ht="30" customHeight="1">
-      <c r="A106" s="105" t="s">
-        <v>746</v>
-      </c>
-      <c r="B106" s="60" t="s">
+      <c r="D107" s="61" t="s">
         <v>766</v>
       </c>
-      <c r="C106" s="61" t="s">
+      <c r="E107" s="61" t="s">
+        <v>495</v>
+      </c>
+      <c r="F107" s="120" t="s">
         <v>767</v>
       </c>
-      <c r="D106" s="61" t="s">
+    </row>
+    <row r="108" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A108" s="106" t="s">
+        <v>744</v>
+      </c>
+      <c r="B108" s="63" t="s">
         <v>768</v>
       </c>
-      <c r="E106" s="61" t="s">
-        <v>495</v>
-      </c>
-      <c r="F106" s="120" t="s">
+      <c r="C108" s="20" t="s">
         <v>769</v>
       </c>
-    </row>
-    <row r="107" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A107" s="106" t="s">
-        <v>746</v>
-      </c>
-      <c r="B107" s="63" t="s">
+      <c r="D108" s="20" t="s">
         <v>770</v>
       </c>
-      <c r="C107" s="20" t="s">
+      <c r="E108" s="20" t="s">
+        <v>551</v>
+      </c>
+      <c r="F108" s="121" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A109" s="109" t="s">
+        <v>744</v>
+      </c>
+      <c r="B109" s="65" t="s">
+        <v>610</v>
+      </c>
+      <c r="C109" s="42" t="s">
         <v>771</v>
       </c>
-      <c r="D107" s="20" t="s">
+      <c r="D109" s="42" t="s">
         <v>772</v>
       </c>
-      <c r="E107" s="20" t="s">
-        <v>553</v>
-      </c>
-      <c r="F107" s="121" t="s">
+      <c r="E109" s="42" t="s">
+        <v>773</v>
+      </c>
+      <c r="F109" s="124" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="108" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A108" s="109" t="s">
-        <v>746</v>
-      </c>
-      <c r="B108" s="65" t="s">
-        <v>612</v>
-      </c>
-      <c r="C108" s="42" t="s">
-        <v>773</v>
-      </c>
-      <c r="D108" s="42" t="s">
+    <row r="110" spans="1:6" ht="30" customHeight="1">
+      <c r="A110" s="99" t="s">
+        <v>744</v>
+      </c>
+      <c r="B110" s="54" t="s">
         <v>774</v>
       </c>
-      <c r="E108" s="42" t="s">
+      <c r="C110" s="15" t="s">
         <v>775</v>
       </c>
-      <c r="F108" s="124" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A109" s="99" t="s">
-        <v>746</v>
-      </c>
-      <c r="B109" s="54" t="s">
+      <c r="D110" s="15" t="s">
         <v>776</v>
       </c>
-      <c r="C109" s="15" t="s">
+      <c r="E110" s="15" t="s">
+        <v>564</v>
+      </c>
+      <c r="F110" s="85" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A111" s="103" t="s">
+        <v>744</v>
+      </c>
+      <c r="B111" s="58" t="s">
         <v>777</v>
       </c>
-      <c r="D109" s="15" t="s">
+      <c r="C111" s="39" t="s">
         <v>778</v>
       </c>
-      <c r="E109" s="15" t="s">
-        <v>566</v>
-      </c>
-      <c r="F109" s="85" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" ht="30" customHeight="1">
-      <c r="A110" s="103" t="s">
-        <v>746</v>
-      </c>
-      <c r="B110" s="58" t="s">
+      <c r="D111" s="39" t="s">
         <v>779</v>
       </c>
-      <c r="C110" s="39" t="s">
+      <c r="E111" s="39" t="s">
         <v>780</v>
       </c>
-      <c r="D110" s="39" t="s">
+      <c r="F111" s="118" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" ht="30" customHeight="1">
+      <c r="A112" s="101" t="s">
+        <v>744</v>
+      </c>
+      <c r="B112" s="56" t="s">
         <v>781</v>
       </c>
-      <c r="E110" s="39" t="s">
+      <c r="C112" s="10" t="s">
         <v>782</v>
       </c>
-      <c r="F110" s="118" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A111" s="101" t="s">
-        <v>746</v>
-      </c>
-      <c r="B111" s="56" t="s">
+      <c r="D112" s="10" t="s">
         <v>783</v>
       </c>
-      <c r="C111" s="10" t="s">
-        <v>784</v>
-      </c>
-      <c r="D111" s="10" t="s">
-        <v>785</v>
-      </c>
-      <c r="E111" s="10" t="s">
-        <v>631</v>
-      </c>
-      <c r="F111" s="116" t="s">
-        <v>710</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" ht="30" customHeight="1">
-      <c r="A112" s="103" t="s">
-        <v>746</v>
-      </c>
-      <c r="B112" s="58" t="s">
-        <v>570</v>
-      </c>
-      <c r="C112" s="39" t="s">
-        <v>786</v>
-      </c>
-      <c r="D112" s="39" t="s">
-        <v>787</v>
-      </c>
-      <c r="E112" s="39" t="s">
-        <v>573</v>
-      </c>
-      <c r="F112" s="118" t="s">
-        <v>353</v>
+      <c r="E112" s="10" t="s">
+        <v>629</v>
+      </c>
+      <c r="F112" s="116" t="s">
+        <v>708</v>
       </c>
     </row>
     <row r="113" spans="1:6" ht="45" customHeight="1">
       <c r="A113" s="103" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="B113" s="58" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="C113" s="39" t="s">
+        <v>784</v>
+      </c>
+      <c r="D113" s="39" t="s">
+        <v>785</v>
+      </c>
+      <c r="E113" s="39" t="s">
+        <v>571</v>
+      </c>
+      <c r="F113" s="118" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A114" s="103" t="s">
+        <v>744</v>
+      </c>
+      <c r="B114" s="58" t="s">
+        <v>568</v>
+      </c>
+      <c r="C114" s="39" t="s">
+        <v>786</v>
+      </c>
+      <c r="D114" s="39" t="s">
+        <v>787</v>
+      </c>
+      <c r="E114" s="39" t="s">
+        <v>571</v>
+      </c>
+      <c r="F114" s="118" t="s">
         <v>788</v>
       </c>
-      <c r="D113" s="39" t="s">
+    </row>
+    <row r="115" spans="1:6" ht="21.75" customHeight="1">
+      <c r="A115" s="104" t="s">
+        <v>744</v>
+      </c>
+      <c r="B115" s="59" t="s">
+        <v>568</v>
+      </c>
+      <c r="C115" s="47" t="s">
         <v>789</v>
       </c>
-      <c r="E113" s="39" t="s">
-        <v>573</v>
-      </c>
-      <c r="F113" s="118" t="s">
+      <c r="D115" s="47" t="s">
         <v>790</v>
       </c>
-    </row>
-    <row r="114" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A114" s="104" t="s">
-        <v>746</v>
-      </c>
-      <c r="B114" s="59" t="s">
-        <v>570</v>
-      </c>
-      <c r="C114" s="47" t="s">
+      <c r="E115" s="47" t="s">
+        <v>571</v>
+      </c>
+      <c r="F115" s="119" t="s">
         <v>791</v>
       </c>
-      <c r="D114" s="47" t="s">
+    </row>
+    <row r="116" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A116" s="166" t="s">
         <v>792</v>
       </c>
-      <c r="E114" s="47" t="s">
-        <v>573</v>
-      </c>
-      <c r="F114" s="119" t="s">
+      <c r="B116" s="167"/>
+      <c r="C116" s="167"/>
+      <c r="D116" s="167"/>
+      <c r="E116" s="167"/>
+      <c r="F116" s="168"/>
+    </row>
+    <row r="117" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A117" s="101" t="s">
         <v>793</v>
       </c>
-    </row>
-    <row r="115" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A115" s="157" t="s">
+      <c r="B117" s="56" t="s">
         <v>794</v>
       </c>
-      <c r="B115" s="158"/>
-      <c r="C115" s="158"/>
-      <c r="D115" s="158"/>
-      <c r="E115" s="158"/>
-      <c r="F115" s="159"/>
-    </row>
-    <row r="116" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A116" s="101" t="s">
+      <c r="C117" s="10" t="s">
+        <v>698</v>
+      </c>
+      <c r="D117" s="10" t="s">
         <v>795</v>
       </c>
-      <c r="B116" s="56" t="s">
-        <v>796</v>
-      </c>
-      <c r="C116" s="10" t="s">
-        <v>700</v>
-      </c>
-      <c r="D116" s="10" t="s">
-        <v>797</v>
-      </c>
-      <c r="E116" s="10" t="s">
-        <v>581</v>
-      </c>
-      <c r="F116" s="116" t="s">
+      <c r="E117" s="10" t="s">
+        <v>579</v>
+      </c>
+      <c r="F117" s="116" t="s">
         <v>37</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A117" s="100" t="s">
-        <v>795</v>
-      </c>
-      <c r="B117" s="55" t="s">
-        <v>798</v>
-      </c>
-      <c r="C117" s="50" t="s">
-        <v>799</v>
-      </c>
-      <c r="D117" s="50" t="s">
-        <v>800</v>
-      </c>
-      <c r="E117" s="50" t="s">
-        <v>709</v>
-      </c>
-      <c r="F117" s="115" t="s">
-        <v>801</v>
       </c>
     </row>
     <row r="118" spans="1:6" ht="30" customHeight="1">
       <c r="A118" s="100" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="B118" s="55" t="s">
-        <v>802</v>
+        <v>796</v>
       </c>
       <c r="C118" s="50" t="s">
-        <v>803</v>
+        <v>797</v>
       </c>
       <c r="D118" s="50" t="s">
-        <v>804</v>
+        <v>798</v>
       </c>
       <c r="E118" s="50" t="s">
-        <v>805</v>
+        <v>707</v>
       </c>
       <c r="F118" s="115" t="s">
-        <v>409</v>
+        <v>799</v>
       </c>
     </row>
     <row r="119" spans="1:6" ht="25.5" customHeight="1">
       <c r="A119" s="100" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="B119" s="55" t="s">
+        <v>800</v>
+      </c>
+      <c r="C119" s="50" t="s">
+        <v>801</v>
+      </c>
+      <c r="D119" s="50" t="s">
+        <v>802</v>
+      </c>
+      <c r="E119" s="50" t="s">
+        <v>803</v>
+      </c>
+      <c r="F119" s="115" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" ht="30" customHeight="1">
+      <c r="A120" s="100" t="s">
+        <v>793</v>
+      </c>
+      <c r="B120" s="55" t="s">
+        <v>804</v>
+      </c>
+      <c r="C120" s="50" t="s">
+        <v>805</v>
+      </c>
+      <c r="D120" s="50" t="s">
         <v>806</v>
       </c>
-      <c r="C119" s="50" t="s">
+      <c r="E120" s="50" t="s">
         <v>807</v>
       </c>
-      <c r="D119" s="50" t="s">
+      <c r="F120" s="115" t="s">
         <v>808</v>
       </c>
-      <c r="E119" s="50" t="s">
+    </row>
+    <row r="121" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A121" s="99" t="s">
+        <v>793</v>
+      </c>
+      <c r="B121" s="54" t="s">
         <v>809</v>
       </c>
-      <c r="F119" s="115" t="s">
+      <c r="C121" s="15" t="s">
         <v>810</v>
       </c>
-    </row>
-    <row r="120" spans="1:6" ht="30" customHeight="1">
-      <c r="A120" s="99" t="s">
-        <v>795</v>
-      </c>
-      <c r="B120" s="54" t="s">
+      <c r="D121" s="15" t="s">
         <v>811</v>
       </c>
-      <c r="C120" s="15" t="s">
+      <c r="E121" s="15" t="s">
+        <v>408</v>
+      </c>
+      <c r="F121" s="85" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A122" s="98" t="s">
+        <v>793</v>
+      </c>
+      <c r="B122" s="53" t="s">
         <v>812</v>
       </c>
-      <c r="D120" s="15" t="s">
+      <c r="C122" s="5" t="s">
         <v>813</v>
       </c>
-      <c r="E120" s="15" t="s">
-        <v>408</v>
-      </c>
-      <c r="F120" s="85" t="s">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A121" s="98" t="s">
-        <v>795</v>
-      </c>
-      <c r="B121" s="53" t="s">
+      <c r="D122" s="5" t="s">
         <v>814</v>
       </c>
-      <c r="C121" s="5" t="s">
+      <c r="E122" s="5" t="s">
         <v>815</v>
       </c>
-      <c r="D121" s="5" t="s">
+      <c r="F122" s="114" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A123" s="99" t="s">
+        <v>793</v>
+      </c>
+      <c r="B123" s="54" t="s">
         <v>816</v>
       </c>
-      <c r="E121" s="5" t="s">
+      <c r="C123" s="15" t="s">
         <v>817</v>
       </c>
-      <c r="F121" s="114" t="s">
-        <v>809</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A122" s="99" t="s">
-        <v>795</v>
-      </c>
-      <c r="B122" s="54" t="s">
+      <c r="D123" s="15" t="s">
         <v>818</v>
       </c>
-      <c r="C122" s="15" t="s">
+      <c r="E123" s="15" t="s">
         <v>819</v>
       </c>
-      <c r="D122" s="15" t="s">
+      <c r="F123" s="113" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" ht="25.5" customHeight="1">
+      <c r="A124" s="98" t="s">
+        <v>793</v>
+      </c>
+      <c r="B124" s="53" t="s">
         <v>820</v>
       </c>
-      <c r="E122" s="15" t="s">
+      <c r="C124" s="5" t="s">
         <v>821</v>
       </c>
-      <c r="F122" s="113" t="s">
-        <v>809</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A123" s="98" t="s">
-        <v>795</v>
-      </c>
-      <c r="B123" s="53" t="s">
+      <c r="D124" s="5" t="s">
         <v>822</v>
       </c>
-      <c r="C123" s="5" t="s">
+      <c r="E124" s="5" t="s">
         <v>823</v>
       </c>
-      <c r="D123" s="5" t="s">
+      <c r="F124" s="114" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" ht="29" thickBot="1">
+      <c r="A125" s="112" t="s">
+        <v>793</v>
+      </c>
+      <c r="B125" s="96" t="s">
+        <v>513</v>
+      </c>
+      <c r="C125" s="97" t="s">
         <v>824</v>
       </c>
-      <c r="E123" s="5" t="s">
+      <c r="D125" s="97" t="s">
         <v>825</v>
       </c>
-      <c r="F123" s="114" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" ht="25.5" customHeight="1" thickBot="1">
-      <c r="A124" s="112" t="s">
-        <v>795</v>
-      </c>
-      <c r="B124" s="96" t="s">
-        <v>515</v>
-      </c>
-      <c r="C124" s="97" t="s">
+      <c r="E125" s="97" t="s">
         <v>826</v>
       </c>
-      <c r="D124" s="97" t="s">
+      <c r="F125" s="127" t="s">
         <v>827</v>
-      </c>
-      <c r="E124" s="97" t="s">
-        <v>828</v>
-      </c>
-      <c r="F124" s="127" t="s">
-        <v>829</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A64:F64"/>
+    <mergeCell ref="A84:F84"/>
+    <mergeCell ref="A100:F100"/>
+    <mergeCell ref="A116:F116"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A48:F48"/>
-    <mergeCell ref="A63:F63"/>
-    <mergeCell ref="A83:F83"/>
-    <mergeCell ref="A99:F99"/>
-    <mergeCell ref="A115:F115"/>
+    <mergeCell ref="A32:F32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18682,13 +18723,13 @@
         <v>53</v>
       </c>
       <c r="B9" s="69" t="s">
+        <v>828</v>
+      </c>
+      <c r="C9" s="67" t="s">
+        <v>829</v>
+      </c>
+      <c r="D9" s="66" t="s">
         <v>830</v>
-      </c>
-      <c r="C9" s="67" t="s">
-        <v>831</v>
-      </c>
-      <c r="D9" s="66" t="s">
-        <v>832</v>
       </c>
       <c r="E9" s="68" t="s">
         <v>185</v>
@@ -18699,13 +18740,13 @@
         <v>53</v>
       </c>
       <c r="B10" s="69" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="C10" s="67" t="s">
         <v>207</v>
       </c>
       <c r="D10" s="66" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="E10" s="68" t="s">
         <v>61</v>
@@ -18861,13 +18902,13 @@
         <v>90</v>
       </c>
       <c r="B21" s="66" t="s">
+        <v>833</v>
+      </c>
+      <c r="C21" s="67" t="s">
+        <v>834</v>
+      </c>
+      <c r="D21" s="66" t="s">
         <v>835</v>
-      </c>
-      <c r="C21" s="67" t="s">
-        <v>836</v>
-      </c>
-      <c r="D21" s="66" t="s">
-        <v>837</v>
       </c>
       <c r="E21" s="68" t="s">
         <v>235</v>
@@ -19057,13 +19098,13 @@
         <v>67</v>
       </c>
       <c r="B34" s="73" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="C34" s="71" t="s">
         <v>273</v>
       </c>
       <c r="D34" s="70" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="E34" s="72" t="s">
         <v>103</v>
@@ -19115,24 +19156,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
-      <c r="A1" s="190" t="s">
-        <v>880</v>
-      </c>
-      <c r="B1" s="191"/>
-      <c r="C1" s="191"/>
-      <c r="D1" s="191"/>
-      <c r="E1" s="191"/>
-      <c r="F1" s="192"/>
-    </row>
-    <row r="2" spans="1:6" ht="21.75" customHeight="1">
-      <c r="A2" s="193" t="s">
-        <v>881</v>
-      </c>
-      <c r="B2" s="194"/>
-      <c r="C2" s="194"/>
-      <c r="D2" s="194"/>
-      <c r="E2" s="194"/>
-      <c r="F2" s="195"/>
+      <c r="A1" s="178" t="s">
+        <v>878</v>
+      </c>
+      <c r="B1" s="179"/>
+      <c r="C1" s="179"/>
+      <c r="D1" s="179"/>
+      <c r="E1" s="179"/>
+      <c r="F1" s="180"/>
+    </row>
+    <row r="2" spans="1:6" ht="34" customHeight="1">
+      <c r="A2" s="181" t="s">
+        <v>879</v>
+      </c>
+      <c r="B2" s="182"/>
+      <c r="C2" s="182"/>
+      <c r="D2" s="182"/>
+      <c r="E2" s="182"/>
+      <c r="F2" s="183"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1">
       <c r="A3" s="77" t="s">
@@ -19155,14 +19196,14 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A4" s="187" t="s">
+      <c r="A4" s="184" t="s">
         <v>146</v>
       </c>
-      <c r="B4" s="188"/>
-      <c r="C4" s="188"/>
-      <c r="D4" s="188"/>
-      <c r="E4" s="188"/>
-      <c r="F4" s="189"/>
+      <c r="B4" s="185"/>
+      <c r="C4" s="185"/>
+      <c r="D4" s="185"/>
+      <c r="E4" s="185"/>
+      <c r="F4" s="186"/>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1">
       <c r="A5" s="78" t="s">
@@ -19226,19 +19267,19 @@
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1">
       <c r="A8" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B8" s="75">
         <v>4.5</v>
       </c>
       <c r="C8" s="76" t="s">
+        <v>839</v>
+      </c>
+      <c r="D8" s="75" t="s">
+        <v>840</v>
+      </c>
+      <c r="E8" s="76" t="s">
         <v>841</v>
-      </c>
-      <c r="D8" s="75" t="s">
-        <v>842</v>
-      </c>
-      <c r="E8" s="76" t="s">
-        <v>843</v>
       </c>
       <c r="F8" s="87" t="s">
         <v>152</v>
@@ -19246,33 +19287,33 @@
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B9" s="68">
         <v>4.5</v>
       </c>
       <c r="C9" s="66" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="D9" s="68" t="s">
         <v>107</v>
       </c>
       <c r="E9" s="66" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="F9" s="88" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A10" s="187" t="s">
+      <c r="A10" s="184" t="s">
         <v>162</v>
       </c>
-      <c r="B10" s="188"/>
-      <c r="C10" s="188"/>
-      <c r="D10" s="188"/>
-      <c r="E10" s="188"/>
-      <c r="F10" s="189"/>
+      <c r="B10" s="185"/>
+      <c r="C10" s="185"/>
+      <c r="D10" s="185"/>
+      <c r="E10" s="185"/>
+      <c r="F10" s="186"/>
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1">
       <c r="A11" s="78" t="s">
@@ -19336,53 +19377,53 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B14" s="75">
         <v>4.8</v>
       </c>
       <c r="C14" s="76" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="D14" s="75" t="s">
         <v>66</v>
       </c>
       <c r="E14" s="76" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="F14" s="87" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="30" customHeight="1">
       <c r="A15" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B15" s="68">
         <v>4.5999999999999996</v>
       </c>
       <c r="C15" s="66" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="D15" s="68" t="s">
         <v>111</v>
       </c>
       <c r="E15" s="66" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="F15" s="88" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A16" s="187" t="s">
+      <c r="A16" s="184" t="s">
         <v>174</v>
       </c>
-      <c r="B16" s="188"/>
-      <c r="C16" s="188"/>
-      <c r="D16" s="188"/>
-      <c r="E16" s="188"/>
-      <c r="F16" s="189"/>
+      <c r="B16" s="185"/>
+      <c r="C16" s="185"/>
+      <c r="D16" s="185"/>
+      <c r="E16" s="185"/>
+      <c r="F16" s="186"/>
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1">
       <c r="A17" s="78" t="s">
@@ -19452,13 +19493,13 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="C20" s="76" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
       <c r="D20" s="75" t="s">
         <v>257</v>
       </c>
       <c r="E20" s="76" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="F20" s="87" t="s">
         <v>303</v>
@@ -19466,33 +19507,33 @@
     </row>
     <row r="21" spans="1:6" ht="30" customHeight="1">
       <c r="A21" s="82" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B21" s="68">
         <v>4.3</v>
       </c>
       <c r="C21" s="66" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="D21" s="68" t="s">
         <v>257</v>
       </c>
       <c r="E21" s="66" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="F21" s="88" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A22" s="187" t="s">
+      <c r="A22" s="184" t="s">
         <v>188</v>
       </c>
-      <c r="B22" s="188"/>
-      <c r="C22" s="188"/>
-      <c r="D22" s="188"/>
-      <c r="E22" s="188"/>
-      <c r="F22" s="189"/>
+      <c r="B22" s="185"/>
+      <c r="C22" s="185"/>
+      <c r="D22" s="185"/>
+      <c r="E22" s="185"/>
+      <c r="F22" s="186"/>
     </row>
     <row r="23" spans="1:6" ht="30" customHeight="1">
       <c r="A23" s="78" t="s">
@@ -19556,53 +19597,53 @@
     </row>
     <row r="26" spans="1:6" ht="30" customHeight="1">
       <c r="A26" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B26" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C26" s="76" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="D26" s="75" t="s">
         <v>160</v>
       </c>
       <c r="E26" s="76" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="F26" s="87" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="30" customHeight="1">
       <c r="A27" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B27" s="68">
         <v>4.4000000000000004</v>
       </c>
       <c r="C27" s="66" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="D27" s="68" t="s">
         <v>220</v>
       </c>
       <c r="E27" s="66" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="F27" s="88" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A28" s="187" t="s">
+      <c r="A28" s="184" t="s">
         <v>201</v>
       </c>
-      <c r="B28" s="188"/>
-      <c r="C28" s="188"/>
-      <c r="D28" s="188"/>
-      <c r="E28" s="188"/>
-      <c r="F28" s="189"/>
+      <c r="B28" s="185"/>
+      <c r="C28" s="185"/>
+      <c r="D28" s="185"/>
+      <c r="E28" s="185"/>
+      <c r="F28" s="186"/>
     </row>
     <row r="29" spans="1:6" ht="30" customHeight="1">
       <c r="A29" s="78" t="s">
@@ -19652,33 +19693,33 @@
         <v>4.3</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="F31" s="86" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="30" customHeight="1">
       <c r="A32" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B32" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C32" s="76" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="D32" s="75" t="s">
         <v>167</v>
       </c>
       <c r="E32" s="76" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="F32" s="87" t="s">
         <v>207</v>
@@ -19686,33 +19727,33 @@
     </row>
     <row r="33" spans="1:6" ht="30" customHeight="1">
       <c r="A33" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B33" s="68">
         <v>4.4000000000000004</v>
       </c>
       <c r="C33" s="66" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="D33" s="68" t="s">
         <v>61</v>
       </c>
       <c r="E33" s="66" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="F33" s="88" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A34" s="184" t="s">
+      <c r="A34" s="187" t="s">
         <v>209</v>
       </c>
-      <c r="B34" s="185"/>
-      <c r="C34" s="185"/>
-      <c r="D34" s="185"/>
-      <c r="E34" s="185"/>
-      <c r="F34" s="186"/>
+      <c r="B34" s="188"/>
+      <c r="C34" s="188"/>
+      <c r="D34" s="188"/>
+      <c r="E34" s="188"/>
+      <c r="F34" s="189"/>
     </row>
     <row r="35" spans="1:6" ht="30" customHeight="1">
       <c r="A35" s="78" t="s">
@@ -19722,16 +19763,16 @@
         <v>4.5</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
       <c r="D35" s="27" t="s">
         <v>220</v>
       </c>
       <c r="E35" s="28" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
       <c r="F35" s="84" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="30" customHeight="1">
@@ -19776,19 +19817,19 @@
     </row>
     <row r="38" spans="1:6" ht="30" customHeight="1">
       <c r="A38" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B38" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C38" s="76" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="D38" s="75" t="s">
         <v>216</v>
       </c>
       <c r="E38" s="76" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="F38" s="87" t="s">
         <v>92</v>
@@ -19796,33 +19837,33 @@
     </row>
     <row r="39" spans="1:6" ht="30" customHeight="1">
       <c r="A39" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B39" s="68">
         <v>4.3</v>
       </c>
       <c r="C39" s="66" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="D39" s="68" t="s">
         <v>224</v>
       </c>
       <c r="E39" s="66" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="F39" s="88" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A40" s="184" t="s">
+      <c r="A40" s="187" t="s">
         <v>218</v>
       </c>
-      <c r="B40" s="185"/>
-      <c r="C40" s="185"/>
-      <c r="D40" s="185"/>
-      <c r="E40" s="185"/>
-      <c r="F40" s="186"/>
+      <c r="B40" s="188"/>
+      <c r="C40" s="188"/>
+      <c r="D40" s="188"/>
+      <c r="E40" s="188"/>
+      <c r="F40" s="189"/>
     </row>
     <row r="41" spans="1:6" ht="30" customHeight="1">
       <c r="A41" s="78" t="s">
@@ -19886,19 +19927,19 @@
     </row>
     <row r="44" spans="1:6" ht="30" customHeight="1">
       <c r="A44" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B44" s="75">
         <v>4.5</v>
       </c>
       <c r="C44" s="76" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="D44" s="75" t="s">
         <v>89</v>
       </c>
       <c r="E44" s="76" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="F44" s="87" t="s">
         <v>226</v>
@@ -19906,33 +19947,33 @@
     </row>
     <row r="45" spans="1:6" ht="30" customHeight="1">
       <c r="A45" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B45" s="68">
         <v>4.4000000000000004</v>
       </c>
       <c r="C45" s="66" t="s">
+        <v>858</v>
+      </c>
+      <c r="D45" s="68" t="s">
+        <v>859</v>
+      </c>
+      <c r="E45" s="66" t="s">
         <v>860</v>
       </c>
-      <c r="D45" s="68" t="s">
+      <c r="F45" s="88" t="s">
         <v>861</v>
       </c>
-      <c r="E45" s="66" t="s">
-        <v>862</v>
-      </c>
-      <c r="F45" s="88" t="s">
-        <v>863</v>
-      </c>
     </row>
     <row r="46" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A46" s="184" t="s">
+      <c r="A46" s="187" t="s">
         <v>230</v>
       </c>
-      <c r="B46" s="185"/>
-      <c r="C46" s="185"/>
-      <c r="D46" s="185"/>
-      <c r="E46" s="185"/>
-      <c r="F46" s="186"/>
+      <c r="B46" s="188"/>
+      <c r="C46" s="188"/>
+      <c r="D46" s="188"/>
+      <c r="E46" s="188"/>
+      <c r="F46" s="189"/>
     </row>
     <row r="47" spans="1:6" ht="30" customHeight="1">
       <c r="A47" s="78" t="s">
@@ -19982,67 +20023,67 @@
         <v>4.5</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>220</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="F49" s="86" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="30" customHeight="1">
       <c r="A50" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B50" s="75">
         <v>4.7</v>
       </c>
       <c r="C50" s="76" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="D50" s="75" t="s">
         <v>66</v>
       </c>
       <c r="E50" s="76" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="F50" s="87" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="30" customHeight="1">
       <c r="A51" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B51" s="68">
         <v>4.4000000000000004</v>
       </c>
       <c r="C51" s="66" t="s">
+        <v>865</v>
+      </c>
+      <c r="D51" s="68" t="s">
+        <v>866</v>
+      </c>
+      <c r="E51" s="66" t="s">
         <v>867</v>
       </c>
-      <c r="D51" s="68" t="s">
+      <c r="F51" s="88" t="s">
         <v>868</v>
       </c>
-      <c r="E51" s="66" t="s">
-        <v>869</v>
-      </c>
-      <c r="F51" s="88" t="s">
-        <v>870</v>
-      </c>
     </row>
     <row r="52" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A52" s="184" t="s">
+      <c r="A52" s="187" t="s">
         <v>238</v>
       </c>
-      <c r="B52" s="185"/>
-      <c r="C52" s="185"/>
-      <c r="D52" s="185"/>
-      <c r="E52" s="185"/>
-      <c r="F52" s="186"/>
+      <c r="B52" s="188"/>
+      <c r="C52" s="188"/>
+      <c r="D52" s="188"/>
+      <c r="E52" s="188"/>
+      <c r="F52" s="189"/>
     </row>
     <row r="53" spans="1:6" ht="30" customHeight="1">
       <c r="A53" s="78" t="s">
@@ -20106,53 +20147,53 @@
     </row>
     <row r="56" spans="1:6" ht="30" customHeight="1">
       <c r="A56" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B56" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C56" s="74" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="D56" s="75" t="s">
         <v>220</v>
       </c>
       <c r="E56" s="76" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="F56" s="87" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="30" customHeight="1">
       <c r="A57" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B57" s="68">
         <v>4.5999999999999996</v>
       </c>
       <c r="C57" s="69" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="D57" s="68" t="s">
         <v>52</v>
       </c>
       <c r="E57" s="66" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="F57" s="88" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A58" s="184" t="s">
+      <c r="A58" s="187" t="s">
         <v>247</v>
       </c>
-      <c r="B58" s="185"/>
-      <c r="C58" s="185"/>
-      <c r="D58" s="185"/>
-      <c r="E58" s="185"/>
-      <c r="F58" s="186"/>
+      <c r="B58" s="188"/>
+      <c r="C58" s="188"/>
+      <c r="D58" s="188"/>
+      <c r="E58" s="188"/>
+      <c r="F58" s="189"/>
     </row>
     <row r="59" spans="1:6" ht="30" customHeight="1">
       <c r="A59" s="78" t="s">
@@ -20215,14 +20256,14 @@
       </c>
     </row>
     <row r="62" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A62" s="178" t="s">
+      <c r="A62" s="190" t="s">
         <v>260</v>
       </c>
-      <c r="B62" s="179"/>
-      <c r="C62" s="179"/>
-      <c r="D62" s="179"/>
-      <c r="E62" s="179"/>
-      <c r="F62" s="180"/>
+      <c r="B62" s="191"/>
+      <c r="C62" s="191"/>
+      <c r="D62" s="191"/>
+      <c r="E62" s="191"/>
+      <c r="F62" s="192"/>
     </row>
     <row r="63" spans="1:6" ht="30" customHeight="1">
       <c r="A63" s="78" t="s">
@@ -20252,13 +20293,13 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="C64" s="16" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="D64" s="18" t="s">
         <v>224</v>
       </c>
       <c r="E64" s="15" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="F64" s="85" t="s">
         <v>279</v>
@@ -20286,19 +20327,19 @@
     </row>
     <row r="66" spans="1:6" ht="30" customHeight="1">
       <c r="A66" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B66" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C66" s="76" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="D66" s="75" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="E66" s="76" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="F66" s="87" t="s">
         <v>279</v>
@@ -20306,39 +20347,39 @@
     </row>
     <row r="67" spans="1:6" ht="30" customHeight="1">
       <c r="A67" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B67" s="68">
         <v>4.3</v>
       </c>
       <c r="C67" s="66" t="s">
+        <v>912</v>
+      </c>
+      <c r="D67" s="68" t="s">
+        <v>913</v>
+      </c>
+      <c r="E67" s="66" t="s">
         <v>914</v>
       </c>
-      <c r="D67" s="68" t="s">
+      <c r="F67" s="88" t="s">
         <v>915</v>
-      </c>
-      <c r="E67" s="66" t="s">
-        <v>916</v>
-      </c>
-      <c r="F67" s="88" t="s">
-        <v>917</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="30" customHeight="1">
       <c r="A68" s="81" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="B68" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C68" s="76" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="D68" s="75" t="s">
         <v>123</v>
       </c>
       <c r="E68" s="76" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="F68" s="87" t="s">
         <v>121</v>
@@ -20346,33 +20387,33 @@
     </row>
     <row r="69" spans="1:6" ht="30" customHeight="1">
       <c r="A69" s="82" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="B69" s="68">
         <v>4.5</v>
       </c>
       <c r="C69" s="66" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="D69" s="68" t="s">
         <v>99</v>
       </c>
       <c r="E69" s="66" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="F69" s="88" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A70" s="178" t="s">
+      <c r="A70" s="190" t="s">
         <v>267</v>
       </c>
-      <c r="B70" s="179"/>
-      <c r="C70" s="179"/>
-      <c r="D70" s="179"/>
-      <c r="E70" s="179"/>
-      <c r="F70" s="180"/>
+      <c r="B70" s="191"/>
+      <c r="C70" s="191"/>
+      <c r="D70" s="191"/>
+      <c r="E70" s="191"/>
+      <c r="F70" s="192"/>
     </row>
     <row r="71" spans="1:6" ht="30" customHeight="1">
       <c r="A71" s="78" t="s">
@@ -20436,19 +20477,19 @@
     </row>
     <row r="74" spans="1:6" ht="30" customHeight="1">
       <c r="A74" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B74" s="75">
         <v>4.3</v>
       </c>
       <c r="C74" s="76" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="D74" s="75" t="s">
         <v>220</v>
       </c>
       <c r="E74" s="76" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="F74" s="87" t="s">
         <v>273</v>
@@ -20456,33 +20497,33 @@
     </row>
     <row r="75" spans="1:6" ht="30" customHeight="1">
       <c r="A75" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B75" s="68">
         <v>4</v>
       </c>
       <c r="C75" s="66" t="s">
+        <v>873</v>
+      </c>
+      <c r="D75" s="68" t="s">
+        <v>874</v>
+      </c>
+      <c r="E75" s="66" t="s">
         <v>875</v>
-      </c>
-      <c r="D75" s="68" t="s">
-        <v>876</v>
-      </c>
-      <c r="E75" s="66" t="s">
-        <v>877</v>
       </c>
       <c r="F75" s="88" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A76" s="178" t="s">
+      <c r="A76" s="190" t="s">
         <v>275</v>
       </c>
-      <c r="B76" s="179"/>
-      <c r="C76" s="179"/>
-      <c r="D76" s="179"/>
-      <c r="E76" s="179"/>
-      <c r="F76" s="180"/>
+      <c r="B76" s="191"/>
+      <c r="C76" s="191"/>
+      <c r="D76" s="191"/>
+      <c r="E76" s="191"/>
+      <c r="F76" s="192"/>
     </row>
     <row r="77" spans="1:6" ht="30" customHeight="1">
       <c r="A77" s="78" t="s">
@@ -20512,13 +20553,13 @@
         <v>4.2</v>
       </c>
       <c r="C78" s="16" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="D78" s="18" t="s">
         <v>119</v>
       </c>
       <c r="E78" s="15" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="F78" s="85" t="s">
         <v>279</v>
@@ -20532,13 +20573,13 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="C79" s="13" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>220</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="F79" s="86" t="s">
         <v>279</v>
@@ -20546,19 +20587,19 @@
     </row>
     <row r="80" spans="1:6" ht="30" customHeight="1">
       <c r="A80" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B80" s="75">
         <v>4.3</v>
       </c>
       <c r="C80" s="76" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="D80" s="75" t="s">
         <v>119</v>
       </c>
       <c r="E80" s="76" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="F80" s="87" t="s">
         <v>279</v>
@@ -20566,19 +20607,19 @@
     </row>
     <row r="81" spans="1:6" ht="30" customHeight="1">
       <c r="A81" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B81" s="68">
         <v>4.4000000000000004</v>
       </c>
       <c r="C81" s="66" t="s">
+        <v>921</v>
+      </c>
+      <c r="D81" s="68" t="s">
+        <v>922</v>
+      </c>
+      <c r="E81" s="66" t="s">
         <v>923</v>
-      </c>
-      <c r="D81" s="68" t="s">
-        <v>924</v>
-      </c>
-      <c r="E81" s="66" t="s">
-        <v>925</v>
       </c>
       <c r="F81" s="88" t="s">
         <v>290</v>
@@ -20586,19 +20627,19 @@
     </row>
     <row r="82" spans="1:6" ht="30" customHeight="1">
       <c r="A82" s="81" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="B82" s="75">
         <v>4.5999999999999996</v>
       </c>
       <c r="C82" s="76" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="D82" s="75" t="s">
         <v>128</v>
       </c>
       <c r="E82" s="76" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="F82" s="87" t="s">
         <v>279</v>
@@ -20606,33 +20647,33 @@
     </row>
     <row r="83" spans="1:6" ht="30" customHeight="1">
       <c r="A83" s="82" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="B83" s="68" t="s">
         <v>255</v>
       </c>
       <c r="C83" s="66" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="D83" s="68" t="s">
         <v>291</v>
       </c>
       <c r="E83" s="66" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="F83" s="88" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A84" s="178" t="s">
+      <c r="A84" s="190" t="s">
         <v>281</v>
       </c>
-      <c r="B84" s="179"/>
-      <c r="C84" s="179"/>
-      <c r="D84" s="179"/>
-      <c r="E84" s="179"/>
-      <c r="F84" s="180"/>
+      <c r="B84" s="191"/>
+      <c r="C84" s="191"/>
+      <c r="D84" s="191"/>
+      <c r="E84" s="191"/>
+      <c r="F84" s="192"/>
     </row>
     <row r="85" spans="1:6" ht="30" customHeight="1">
       <c r="A85" s="78" t="s">
@@ -20696,66 +20737,56 @@
     </row>
     <row r="88" spans="1:6" ht="30" customHeight="1">
       <c r="A88" s="81" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B88" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C88" s="76" t="s">
+        <v>924</v>
+      </c>
+      <c r="D88" s="75" t="s">
+        <v>925</v>
+      </c>
+      <c r="E88" s="76" t="s">
         <v>926</v>
       </c>
-      <c r="D88" s="75" t="s">
+      <c r="F88" s="87" t="s">
         <v>927</v>
-      </c>
-      <c r="E88" s="76" t="s">
-        <v>928</v>
-      </c>
-      <c r="F88" s="87" t="s">
-        <v>929</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="30" customHeight="1">
       <c r="A89" s="82" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B89" s="68">
         <v>4.5</v>
       </c>
       <c r="C89" s="66" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="D89" s="68" t="s">
         <v>119</v>
       </c>
       <c r="E89" s="66" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="F89" s="88" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="33.75" customHeight="1" thickBot="1">
-      <c r="A90" s="181" t="s">
-        <v>941</v>
-      </c>
-      <c r="B90" s="182"/>
-      <c r="C90" s="182"/>
-      <c r="D90" s="182"/>
-      <c r="E90" s="182"/>
-      <c r="F90" s="183"/>
+      <c r="A90" s="193" t="s">
+        <v>939</v>
+      </c>
+      <c r="B90" s="194"/>
+      <c r="C90" s="194"/>
+      <c r="D90" s="194"/>
+      <c r="E90" s="194"/>
+      <c r="F90" s="195"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="A46:F46"/>
     <mergeCell ref="A84:F84"/>
     <mergeCell ref="A90:F90"/>
     <mergeCell ref="A52:F52"/>
@@ -20763,6 +20794,16 @@
     <mergeCell ref="A62:F62"/>
     <mergeCell ref="A70:F70"/>
     <mergeCell ref="A76:F76"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A16:F16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -20784,12 +20825,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25.5" customHeight="1">
-      <c r="A1" s="160" t="s">
+      <c r="A1" s="151" t="s">
         <v>292</v>
       </c>
-      <c r="B1" s="161"/>
-      <c r="C1" s="161"/>
-      <c r="D1" s="162"/>
+      <c r="B1" s="152"/>
+      <c r="C1" s="152"/>
+      <c r="D1" s="153"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="132"/>
@@ -20894,13 +20935,13 @@
         <v>326</v>
       </c>
       <c r="B10" s="92" t="s">
+        <v>969</v>
+      </c>
+      <c r="C10" s="92" t="s">
+        <v>970</v>
+      </c>
+      <c r="D10" s="125" t="s">
         <v>971</v>
-      </c>
-      <c r="C10" s="92" t="s">
-        <v>972</v>
-      </c>
-      <c r="D10" s="125" t="s">
-        <v>973</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -21020,27 +21061,27 @@
         <v>326</v>
       </c>
       <c r="B20" s="92" t="s">
+        <v>972</v>
+      </c>
+      <c r="C20" s="92" t="s">
+        <v>973</v>
+      </c>
+      <c r="D20" s="125" t="s">
         <v>974</v>
-      </c>
-      <c r="C20" s="92" t="s">
-        <v>975</v>
-      </c>
-      <c r="D20" s="125" t="s">
-        <v>976</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="30" customHeight="1">
       <c r="A21" s="140" t="s">
+        <v>975</v>
+      </c>
+      <c r="B21" s="90" t="s">
+        <v>976</v>
+      </c>
+      <c r="C21" s="90" t="s">
         <v>977</v>
       </c>
-      <c r="B21" s="90" t="s">
+      <c r="D21" s="149" t="s">
         <v>978</v>
-      </c>
-      <c r="C21" s="90" t="s">
-        <v>979</v>
-      </c>
-      <c r="D21" s="149" t="s">
-        <v>980</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="27.75" customHeight="1">

</xml_diff>